<commit_message>
Updated models data sheet, added second version of Letter_T, added texture template & verts
</commit_message>
<xml_diff>
--- a/letter_graphics/Letter_T_Model_Data.xlsx
+++ b/letter_graphics/Letter_T_Model_Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mtuireland-my.sharepoint.com/personal/t00271915_mymtu_ie/Documents/Computer Graphics/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\StudentMariTarasova(\Documents\GitHub\computer-graphics\letter_graphics\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="50" documentId="8_{3F581A1D-95FE-401E-ADF5-2383C9189251}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{90FB9699-D536-47C4-8A42-92D2B6B8A046}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94C81113-CE69-41C1-8523-5663691C3F57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{B2B28E4F-1194-47DF-9BFD-E244446D9772}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B2B28E4F-1194-47DF-9BFD-E244446D9772}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="14">
   <si>
     <t>x</t>
   </si>
@@ -62,14 +62,32 @@
     <t>2D Verts Back Face</t>
   </si>
   <si>
-    <t>2D Verts Left Face</t>
+    <t>Texture Faces</t>
+  </si>
+  <si>
+    <t>Px</t>
+  </si>
+  <si>
+    <t>Py</t>
+  </si>
+  <si>
+    <t>2D Texture Verts Raw</t>
+  </si>
+  <si>
+    <t>Front Face</t>
+  </si>
+  <si>
+    <t>Back Face</t>
+  </si>
+  <si>
+    <t>Left Face</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -93,7 +111,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="36">
+  <borders count="40">
     <border>
       <left/>
       <right/>
@@ -470,14 +488,53 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="dotted">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
@@ -492,7 +549,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
@@ -501,47 +558,38 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
@@ -553,40 +601,37 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
@@ -605,20 +650,80 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="32" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="37" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="38" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2138,6 +2243,107 @@
     </mc:AlternateContent>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>68</xdr:col>
+      <xdr:colOff>11205</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>11208</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>94</xdr:col>
+      <xdr:colOff>183776</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>183779</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{20F517E5-B645-4FEE-91C0-E6C94F486BE3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="13032440" y="201708"/>
+          <a:ext cx="5125571" cy="5125571"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>156884</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>179294</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>89647</xdr:colOff>
+      <xdr:row>42</xdr:row>
+      <xdr:rowOff>190393</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 13">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6211ED18-5D87-6B96-02AC-3AAD7E5B6CD8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect r="49754" b="43539"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="347384" y="5322794"/>
+          <a:ext cx="4538381" cy="2868599"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -3132,1396 +3338,2854 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A45E7990-8E98-4590-89B6-0D65C03B4C6C}">
-  <dimension ref="B1:AU40"/>
-  <sheetFormatPr defaultColWidth="2.5" defaultRowHeight="15" customHeight="1"/>
+  <dimension ref="B1:BM63"/>
+  <sheetFormatPr defaultColWidth="2.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="14" max="14" width="2.875" bestFit="1" customWidth="1"/>
+    <col min="60" max="60" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:47" ht="15" customHeight="1">
-      <c r="C1" s="2"/>
-      <c r="I1" s="2"/>
+    <row r="1" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="AB1" s="5"/>
+      <c r="AC1" s="5"/>
+      <c r="AD1" s="5"/>
+      <c r="AE1" s="5"/>
+      <c r="AF1" s="5"/>
+      <c r="AG1" s="5"/>
+      <c r="AH1" s="5"/>
+      <c r="AI1" s="5"/>
     </row>
-    <row r="2" spans="2:47" ht="15" customHeight="1">
-      <c r="B2" s="2"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="18"/>
-      <c r="N2" s="34" t="s">
+    <row r="2" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C2" s="2"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="17"/>
+      <c r="N2" s="57" t="s">
         <v>2</v>
       </c>
-      <c r="O2" s="35"/>
-      <c r="P2" s="35"/>
-      <c r="Q2" s="35"/>
-      <c r="R2" s="35"/>
-      <c r="S2" s="36"/>
-      <c r="T2" s="56" t="s">
+      <c r="O2" s="58"/>
+      <c r="P2" s="58"/>
+      <c r="Q2" s="58"/>
+      <c r="R2" s="58"/>
+      <c r="S2" s="59"/>
+      <c r="T2" s="30" t="s">
         <v>3</v>
       </c>
-      <c r="U2" s="35"/>
-      <c r="V2" s="35"/>
-      <c r="W2" s="35"/>
-      <c r="X2" s="35"/>
-      <c r="Y2" s="36"/>
-      <c r="AB2" s="22" t="s">
+      <c r="U2" s="31"/>
+      <c r="V2" s="31"/>
+      <c r="W2" s="31"/>
+      <c r="X2" s="31"/>
+      <c r="Y2" s="32"/>
+      <c r="AA2" s="74"/>
+      <c r="AB2" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="AC2" s="22"/>
-      <c r="AD2" s="22"/>
-      <c r="AE2" s="22"/>
-      <c r="AF2" s="22"/>
-      <c r="AG2" s="22"/>
-      <c r="AH2" s="22"/>
-      <c r="AI2" s="22"/>
+      <c r="AC2" s="31"/>
+      <c r="AD2" s="31"/>
+      <c r="AE2" s="31"/>
+      <c r="AF2" s="31"/>
+      <c r="AG2" s="31"/>
+      <c r="AH2" s="31"/>
+      <c r="AI2" s="32"/>
+      <c r="AL2" s="24" t="s">
+        <v>7</v>
+      </c>
+      <c r="AM2" s="24"/>
+      <c r="AN2" s="24"/>
+      <c r="AO2" s="24"/>
+      <c r="AP2" s="24"/>
+      <c r="AQ2" s="24"/>
+      <c r="AR2" s="24"/>
+      <c r="AS2" s="24"/>
+      <c r="BH2" s="24" t="s">
+        <v>10</v>
+      </c>
+      <c r="BI2" s="24"/>
+      <c r="BJ2" s="24"/>
+      <c r="BK2" s="24"/>
+      <c r="BL2" s="24"/>
+      <c r="BM2" s="24"/>
     </row>
-    <row r="3" spans="2:47" ht="15" customHeight="1">
-      <c r="B3" s="2"/>
+    <row r="3" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C3" s="1"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="17"/>
-      <c r="N3" s="48"/>
-      <c r="O3" s="49"/>
-      <c r="P3" s="39" t="s">
+      <c r="M3" s="16"/>
+      <c r="N3" s="41"/>
+      <c r="O3" s="42"/>
+      <c r="P3" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="Q3" s="38"/>
-      <c r="R3" s="39" t="s">
+      <c r="Q3" s="26"/>
+      <c r="R3" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="S3" s="41"/>
-      <c r="T3" s="37" t="s">
+      <c r="S3" s="27"/>
+      <c r="T3" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="U3" s="38"/>
-      <c r="V3" s="39" t="s">
+      <c r="U3" s="26"/>
+      <c r="V3" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="W3" s="40"/>
-      <c r="X3" s="39" t="s">
+      <c r="W3" s="34"/>
+      <c r="X3" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="Y3" s="41"/>
-      <c r="AB3" s="23"/>
-      <c r="AC3" s="24"/>
-      <c r="AD3" s="22"/>
-      <c r="AE3" s="22"/>
-      <c r="AF3" s="22"/>
-      <c r="AG3" s="22"/>
-      <c r="AH3" s="22"/>
-      <c r="AI3" s="22"/>
+      <c r="Y3" s="27"/>
+      <c r="AA3" s="74"/>
+      <c r="AB3" s="53" t="s">
+        <v>11</v>
+      </c>
+      <c r="AC3" s="54"/>
+      <c r="AD3" s="54"/>
+      <c r="AE3" s="54"/>
+      <c r="AF3" s="54"/>
+      <c r="AG3" s="54"/>
+      <c r="AH3" s="54"/>
+      <c r="AI3" s="55"/>
+      <c r="AL3" s="71"/>
+      <c r="AM3" s="49"/>
+      <c r="AN3" s="71"/>
+      <c r="AO3" s="71"/>
+      <c r="AP3" s="71"/>
+      <c r="AQ3" s="71"/>
+      <c r="AR3" s="71"/>
+      <c r="AS3" s="71"/>
+      <c r="BH3" s="71"/>
+      <c r="BI3" s="49"/>
+      <c r="BJ3" s="72" t="s">
+        <v>8</v>
+      </c>
+      <c r="BK3" s="73"/>
+      <c r="BL3" s="71" t="s">
+        <v>9</v>
+      </c>
+      <c r="BM3" s="71"/>
     </row>
-    <row r="4" spans="2:47" ht="15" customHeight="1" thickBot="1">
-      <c r="B4" s="2"/>
+    <row r="4" spans="3:65" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C4" s="1"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2">
+      <c r="E4">
         <v>0</v>
       </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="15">
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="14">
         <v>1</v>
       </c>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="17"/>
-      <c r="N4" s="42">
+      <c r="M4" s="16"/>
+      <c r="N4" s="20">
         <v>0</v>
       </c>
-      <c r="O4" s="43"/>
-      <c r="P4" s="42">
+      <c r="O4" s="21"/>
+      <c r="P4" s="20">
         <v>-2</v>
       </c>
-      <c r="Q4" s="43"/>
-      <c r="R4" s="42">
+      <c r="Q4" s="21"/>
+      <c r="R4" s="20">
         <v>4</v>
       </c>
-      <c r="S4" s="44"/>
-      <c r="T4" s="57">
+      <c r="S4" s="28"/>
+      <c r="T4" s="35">
         <v>-2</v>
       </c>
-      <c r="U4" s="58"/>
-      <c r="V4" s="59">
+      <c r="U4" s="36"/>
+      <c r="V4" s="37">
         <v>4</v>
       </c>
-      <c r="W4" s="58"/>
-      <c r="X4" s="27">
+      <c r="W4" s="36"/>
+      <c r="X4" s="38">
         <v>1</v>
       </c>
-      <c r="Y4" s="30"/>
-      <c r="AB4" s="23">
+      <c r="Y4" s="39"/>
+      <c r="AA4" s="74"/>
+      <c r="AB4" s="50">
         <v>0</v>
       </c>
-      <c r="AC4" s="24"/>
-      <c r="AD4" s="22">
+      <c r="AC4" s="44"/>
+      <c r="AD4" s="79">
         <v>0</v>
       </c>
-      <c r="AE4" s="22"/>
-      <c r="AF4" s="22">
+      <c r="AE4" s="56"/>
+      <c r="AF4" s="38">
         <v>2</v>
       </c>
-      <c r="AG4" s="22"/>
-      <c r="AH4" s="22">
+      <c r="AG4" s="56"/>
+      <c r="AH4" s="70">
         <v>4</v>
       </c>
-      <c r="AI4" s="22"/>
-      <c r="AP4" s="2"/>
-      <c r="AQ4" s="7"/>
-      <c r="AR4" s="7"/>
-      <c r="AS4" s="7"/>
-      <c r="AT4" s="7"/>
-      <c r="AU4" s="2"/>
+      <c r="AI4" s="44"/>
+      <c r="AL4" s="24"/>
+      <c r="AM4" s="44"/>
+      <c r="AN4" s="24"/>
+      <c r="AO4" s="24"/>
+      <c r="AP4" s="24"/>
+      <c r="AQ4" s="24"/>
+      <c r="AR4" s="24"/>
+      <c r="AS4" s="24"/>
+      <c r="BH4" s="70">
+        <v>0</v>
+      </c>
+      <c r="BI4" s="44"/>
+      <c r="BJ4" s="50"/>
+      <c r="BK4" s="52"/>
+      <c r="BL4" s="24"/>
+      <c r="BM4" s="24"/>
     </row>
-    <row r="5" spans="2:47" ht="15" customHeight="1">
-      <c r="B5" s="2"/>
+    <row r="5" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C5" s="1"/>
-      <c r="D5" s="2">
+      <c r="D5">
         <v>2</v>
       </c>
-      <c r="E5" s="8"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="9"/>
-      <c r="K5" s="15">
+      <c r="E5" s="7"/>
+      <c r="J5" s="8"/>
+      <c r="K5" s="14">
         <v>3</v>
       </c>
-      <c r="L5" s="2"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="42">
+      <c r="M5" s="16"/>
+      <c r="N5" s="20">
         <v>1</v>
       </c>
-      <c r="O5" s="43"/>
-      <c r="P5" s="42">
+      <c r="O5" s="21"/>
+      <c r="P5" s="20">
         <v>2</v>
       </c>
-      <c r="Q5" s="43"/>
-      <c r="R5" s="42">
+      <c r="Q5" s="21"/>
+      <c r="R5" s="20">
         <v>4</v>
       </c>
-      <c r="S5" s="44"/>
-      <c r="T5" s="55">
+      <c r="S5" s="28"/>
+      <c r="T5" s="40">
         <v>2</v>
       </c>
-      <c r="U5" s="43"/>
-      <c r="V5" s="42">
+      <c r="U5" s="21"/>
+      <c r="V5" s="20">
         <v>4</v>
       </c>
-      <c r="W5" s="43"/>
-      <c r="X5" s="25">
+      <c r="W5" s="21"/>
+      <c r="X5" s="43">
         <v>1</v>
       </c>
-      <c r="Y5" s="24"/>
-      <c r="AB5" s="23">
+      <c r="Y5" s="44"/>
+      <c r="AA5" s="74"/>
+      <c r="AB5" s="50">
         <v>1</v>
       </c>
-      <c r="AC5" s="24"/>
-      <c r="AD5" s="22">
+      <c r="AC5" s="44"/>
+      <c r="AD5" s="50">
         <v>0</v>
       </c>
-      <c r="AE5" s="22"/>
-      <c r="AF5" s="22">
+      <c r="AE5" s="52"/>
+      <c r="AF5" s="43">
         <v>4</v>
       </c>
-      <c r="AG5" s="22"/>
-      <c r="AH5" s="22">
+      <c r="AG5" s="52"/>
+      <c r="AH5" s="70">
         <v>1</v>
       </c>
-      <c r="AI5" s="22"/>
-      <c r="AP5" s="8"/>
-      <c r="AQ5" s="2"/>
-      <c r="AR5" s="2"/>
-      <c r="AS5" s="2"/>
-      <c r="AT5" s="2"/>
-      <c r="AU5" s="9"/>
+      <c r="AI5" s="44"/>
+      <c r="AL5" s="24"/>
+      <c r="AM5" s="44"/>
+      <c r="AN5" s="24"/>
+      <c r="AO5" s="24"/>
+      <c r="AP5" s="24"/>
+      <c r="AQ5" s="24"/>
+      <c r="AR5" s="24"/>
+      <c r="AS5" s="24"/>
+      <c r="BH5" s="70">
+        <v>1</v>
+      </c>
+      <c r="BI5" s="44"/>
+      <c r="BJ5" s="50"/>
+      <c r="BK5" s="52"/>
+      <c r="BL5" s="24"/>
+      <c r="BM5" s="24"/>
     </row>
-    <row r="6" spans="2:47" ht="15" customHeight="1" thickBot="1">
-      <c r="B6" s="2"/>
+    <row r="6" spans="3:65" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="C6" s="1"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="9"/>
-      <c r="F6" s="7">
+      <c r="E6" s="8"/>
+      <c r="F6" s="6">
         <v>5</v>
       </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="16">
+      <c r="I6" s="15">
         <v>6</v>
       </c>
-      <c r="J6" s="8"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="17"/>
-      <c r="N6" s="42">
+      <c r="J6" s="7"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="20">
         <v>2</v>
       </c>
-      <c r="O6" s="43"/>
-      <c r="P6" s="42">
+      <c r="O6" s="21"/>
+      <c r="P6" s="20">
         <v>-3</v>
       </c>
-      <c r="Q6" s="43"/>
-      <c r="R6" s="42">
+      <c r="Q6" s="21"/>
+      <c r="R6" s="20">
         <v>3</v>
       </c>
-      <c r="S6" s="44"/>
-      <c r="T6" s="55">
+      <c r="S6" s="28"/>
+      <c r="T6" s="40">
         <v>-3</v>
       </c>
-      <c r="U6" s="43"/>
-      <c r="V6" s="42">
+      <c r="U6" s="21"/>
+      <c r="V6" s="20">
         <v>3</v>
       </c>
-      <c r="W6" s="43"/>
-      <c r="X6" s="25">
+      <c r="W6" s="21"/>
+      <c r="X6" s="43">
         <v>1</v>
       </c>
-      <c r="Y6" s="24"/>
-      <c r="AB6" s="23">
+      <c r="Y6" s="44"/>
+      <c r="AA6" s="74"/>
+      <c r="AB6" s="50">
         <v>2</v>
       </c>
-      <c r="AC6" s="24"/>
-      <c r="AD6" s="22">
+      <c r="AC6" s="44"/>
+      <c r="AD6" s="50">
         <v>1</v>
       </c>
-      <c r="AE6" s="22"/>
-      <c r="AF6" s="22">
+      <c r="AE6" s="52"/>
+      <c r="AF6" s="43">
         <v>4</v>
       </c>
-      <c r="AG6" s="22"/>
-      <c r="AH6" s="22">
+      <c r="AG6" s="52"/>
+      <c r="AH6" s="70">
         <v>7</v>
       </c>
-      <c r="AI6" s="22"/>
-      <c r="AP6" s="9"/>
-      <c r="AQ6" s="7"/>
-      <c r="AR6" s="2"/>
-      <c r="AS6" s="2"/>
-      <c r="AT6" s="7"/>
-      <c r="AU6" s="8"/>
+      <c r="AI6" s="44"/>
+      <c r="AL6" s="24"/>
+      <c r="AM6" s="44"/>
+      <c r="AN6" s="24"/>
+      <c r="AO6" s="24"/>
+      <c r="AP6" s="24"/>
+      <c r="AQ6" s="24"/>
+      <c r="AR6" s="24"/>
+      <c r="AS6" s="24"/>
+      <c r="BH6" s="70">
+        <v>2</v>
+      </c>
+      <c r="BI6" s="44"/>
+      <c r="BJ6" s="50"/>
+      <c r="BK6" s="52"/>
+      <c r="BL6" s="24"/>
+      <c r="BM6" s="24"/>
     </row>
-    <row r="7" spans="2:47" ht="15" customHeight="1">
-      <c r="B7" s="2"/>
+    <row r="7" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C7" s="1"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2">
+      <c r="E7">
         <v>4</v>
       </c>
-      <c r="F7" s="10"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="12"/>
-      <c r="J7" s="15">
+      <c r="F7" s="9"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="14">
         <v>7</v>
       </c>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="17"/>
-      <c r="N7" s="42">
+      <c r="M7" s="16"/>
+      <c r="N7" s="20">
         <v>3</v>
       </c>
-      <c r="O7" s="43"/>
-      <c r="P7" s="42">
+      <c r="O7" s="21"/>
+      <c r="P7" s="20">
         <v>3</v>
       </c>
-      <c r="Q7" s="43"/>
-      <c r="R7" s="42">
+      <c r="Q7" s="21"/>
+      <c r="R7" s="20">
         <v>3</v>
       </c>
-      <c r="S7" s="44"/>
-      <c r="T7" s="55">
+      <c r="S7" s="28"/>
+      <c r="T7" s="40">
         <v>3</v>
       </c>
-      <c r="U7" s="43"/>
-      <c r="V7" s="42">
+      <c r="U7" s="21"/>
+      <c r="V7" s="20">
         <v>3</v>
       </c>
-      <c r="W7" s="43"/>
-      <c r="X7" s="25">
+      <c r="W7" s="21"/>
+      <c r="X7" s="43">
         <v>1</v>
       </c>
-      <c r="Y7" s="24"/>
-      <c r="AB7" s="23">
+      <c r="Y7" s="44"/>
+      <c r="AA7" s="74"/>
+      <c r="AB7" s="50">
         <v>3</v>
       </c>
-      <c r="AC7" s="24"/>
-      <c r="AD7" s="22">
+      <c r="AC7" s="44"/>
+      <c r="AD7" s="50">
         <v>1</v>
       </c>
-      <c r="AE7" s="22"/>
-      <c r="AF7" s="22">
+      <c r="AE7" s="52"/>
+      <c r="AF7" s="43">
         <v>7</v>
       </c>
-      <c r="AG7" s="22"/>
-      <c r="AH7" s="22">
+      <c r="AG7" s="52"/>
+      <c r="AH7" s="70">
         <v>3</v>
       </c>
-      <c r="AI7" s="22"/>
-      <c r="AP7" s="2"/>
-      <c r="AQ7" s="10"/>
-      <c r="AR7" s="2"/>
-      <c r="AS7" s="2"/>
-      <c r="AT7" s="12"/>
-      <c r="AU7" s="2"/>
+      <c r="AI7" s="44"/>
+      <c r="AL7" s="24"/>
+      <c r="AM7" s="44"/>
+      <c r="AN7" s="24"/>
+      <c r="AO7" s="24"/>
+      <c r="AP7" s="24"/>
+      <c r="AQ7" s="24"/>
+      <c r="AR7" s="24"/>
+      <c r="AS7" s="24"/>
+      <c r="BH7" s="70">
+        <v>3</v>
+      </c>
+      <c r="BI7" s="44"/>
+      <c r="BJ7" s="50"/>
+      <c r="BK7" s="52"/>
+      <c r="BL7" s="24"/>
+      <c r="BM7" s="24"/>
     </row>
-    <row r="8" spans="2:47" ht="15" customHeight="1">
-      <c r="B8" s="2"/>
+    <row r="8" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C8" s="1"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="11"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="13"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="17"/>
-      <c r="N8" s="42">
+      <c r="F8" s="10"/>
+      <c r="I8" s="12"/>
+      <c r="M8" s="16"/>
+      <c r="N8" s="20">
         <v>4</v>
       </c>
-      <c r="O8" s="43"/>
-      <c r="P8" s="42">
+      <c r="O8" s="21"/>
+      <c r="P8" s="20">
         <v>-2</v>
       </c>
-      <c r="Q8" s="43"/>
-      <c r="R8" s="42">
+      <c r="Q8" s="21"/>
+      <c r="R8" s="20">
         <v>2</v>
       </c>
-      <c r="S8" s="44"/>
-      <c r="T8" s="55">
+      <c r="S8" s="28"/>
+      <c r="T8" s="40">
         <v>-2</v>
       </c>
-      <c r="U8" s="43"/>
-      <c r="V8" s="42">
+      <c r="U8" s="21"/>
+      <c r="V8" s="20">
         <v>2</v>
       </c>
-      <c r="W8" s="43"/>
-      <c r="X8" s="25">
+      <c r="W8" s="21"/>
+      <c r="X8" s="43">
         <v>1</v>
       </c>
-      <c r="Y8" s="24"/>
-      <c r="AB8" s="23">
+      <c r="Y8" s="44"/>
+      <c r="AA8" s="74"/>
+      <c r="AB8" s="50">
         <v>4</v>
       </c>
-      <c r="AC8" s="24"/>
-      <c r="AD8" s="22"/>
-      <c r="AE8" s="22"/>
-      <c r="AF8" s="22"/>
-      <c r="AG8" s="22"/>
-      <c r="AH8" s="22"/>
-      <c r="AI8" s="22"/>
-      <c r="AP8" s="2"/>
-      <c r="AQ8" s="11"/>
-      <c r="AR8" s="2"/>
-      <c r="AS8" s="2"/>
-      <c r="AT8" s="13"/>
-      <c r="AU8" s="2"/>
+      <c r="AC8" s="44"/>
+      <c r="AD8" s="50">
+        <v>5</v>
+      </c>
+      <c r="AE8" s="52"/>
+      <c r="AF8" s="43">
+        <v>9</v>
+      </c>
+      <c r="AG8" s="52"/>
+      <c r="AH8" s="70">
+        <v>6</v>
+      </c>
+      <c r="AI8" s="44"/>
+      <c r="AL8" s="24"/>
+      <c r="AM8" s="44"/>
+      <c r="AN8" s="24"/>
+      <c r="AO8" s="24"/>
+      <c r="AP8" s="24"/>
+      <c r="AQ8" s="24"/>
+      <c r="AR8" s="24"/>
+      <c r="AS8" s="24"/>
+      <c r="BH8" s="70">
+        <v>4</v>
+      </c>
+      <c r="BI8" s="44"/>
+      <c r="BJ8" s="50"/>
+      <c r="BK8" s="52"/>
+      <c r="BL8" s="24"/>
+      <c r="BM8" s="24"/>
     </row>
-    <row r="9" spans="2:47" ht="15" customHeight="1">
-      <c r="B9" s="2"/>
+    <row r="9" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C9" s="1"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="11"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="13"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="17"/>
-      <c r="N9" s="42">
+      <c r="F9" s="10"/>
+      <c r="I9" s="12"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="20">
         <v>5</v>
       </c>
-      <c r="O9" s="43"/>
-      <c r="P9" s="42">
+      <c r="O9" s="21"/>
+      <c r="P9" s="20">
         <v>-1</v>
       </c>
-      <c r="Q9" s="43"/>
-      <c r="R9" s="42">
+      <c r="Q9" s="21"/>
+      <c r="R9" s="20">
         <v>2</v>
       </c>
-      <c r="S9" s="44"/>
-      <c r="T9" s="55">
+      <c r="S9" s="28"/>
+      <c r="T9" s="40">
         <v>-1</v>
       </c>
-      <c r="U9" s="43"/>
-      <c r="V9" s="42">
+      <c r="U9" s="21"/>
+      <c r="V9" s="20">
         <v>2</v>
       </c>
-      <c r="W9" s="43"/>
-      <c r="X9" s="25">
+      <c r="W9" s="21"/>
+      <c r="X9" s="43">
         <v>1</v>
       </c>
-      <c r="Y9" s="24"/>
-      <c r="AB9" s="23">
+      <c r="Y9" s="44"/>
+      <c r="AA9" s="74"/>
+      <c r="AB9" s="50">
         <v>5</v>
       </c>
-      <c r="AC9" s="24"/>
-      <c r="AD9" s="22"/>
-      <c r="AE9" s="22"/>
-      <c r="AF9" s="22"/>
-      <c r="AG9" s="22"/>
-      <c r="AH9" s="22"/>
-      <c r="AI9" s="22"/>
-      <c r="AP9" s="2"/>
-      <c r="AQ9" s="11"/>
-      <c r="AR9" s="2"/>
-      <c r="AS9" s="2"/>
-      <c r="AT9" s="13"/>
-      <c r="AU9" s="2"/>
+      <c r="AC9" s="44"/>
+      <c r="AD9" s="50">
+        <v>5</v>
+      </c>
+      <c r="AE9" s="52"/>
+      <c r="AF9" s="43">
+        <v>8</v>
+      </c>
+      <c r="AG9" s="52"/>
+      <c r="AH9" s="70">
+        <v>9</v>
+      </c>
+      <c r="AI9" s="44"/>
+      <c r="AL9" s="24"/>
+      <c r="AM9" s="44"/>
+      <c r="AN9" s="24"/>
+      <c r="AO9" s="24"/>
+      <c r="AP9" s="24"/>
+      <c r="AQ9" s="24"/>
+      <c r="AR9" s="24"/>
+      <c r="AS9" s="24"/>
+      <c r="BH9" s="70">
+        <v>5</v>
+      </c>
+      <c r="BI9" s="44"/>
+      <c r="BJ9" s="50"/>
+      <c r="BK9" s="52"/>
+      <c r="BL9" s="24"/>
+      <c r="BM9" s="24"/>
     </row>
-    <row r="10" spans="2:47" ht="15" customHeight="1">
+    <row r="10" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="11"/>
-      <c r="G10" s="2"/>
-      <c r="H10" s="2"/>
-      <c r="I10" s="13"/>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="17"/>
-      <c r="N10" s="42">
+      <c r="F10" s="10"/>
+      <c r="I10" s="12"/>
+      <c r="M10" s="16"/>
+      <c r="N10" s="20">
         <v>6</v>
       </c>
-      <c r="O10" s="43"/>
-      <c r="P10" s="42">
+      <c r="O10" s="21"/>
+      <c r="P10" s="20">
         <v>1</v>
       </c>
-      <c r="Q10" s="43"/>
-      <c r="R10" s="42">
+      <c r="Q10" s="21"/>
+      <c r="R10" s="20">
         <v>2</v>
       </c>
-      <c r="S10" s="44"/>
-      <c r="T10" s="55">
+      <c r="S10" s="28"/>
+      <c r="T10" s="40">
         <v>1</v>
       </c>
-      <c r="U10" s="43"/>
-      <c r="V10" s="42">
+      <c r="U10" s="21"/>
+      <c r="V10" s="20">
         <v>2</v>
       </c>
-      <c r="W10" s="43"/>
-      <c r="X10" s="25">
+      <c r="W10" s="21"/>
+      <c r="X10" s="43">
         <v>1</v>
       </c>
-      <c r="Y10" s="24"/>
-      <c r="AB10" s="23">
+      <c r="Y10" s="44"/>
+      <c r="AA10" s="74"/>
+      <c r="AB10" s="72">
         <v>6</v>
       </c>
-      <c r="AC10" s="24"/>
-      <c r="AD10" s="22"/>
-      <c r="AE10" s="22"/>
-      <c r="AF10" s="22"/>
-      <c r="AG10" s="22"/>
-      <c r="AH10" s="22"/>
-      <c r="AI10" s="22"/>
-      <c r="AQ10" s="11"/>
-      <c r="AR10" s="2"/>
-      <c r="AS10" s="2"/>
-      <c r="AT10" s="13"/>
+      <c r="AC10" s="49"/>
+      <c r="AD10" s="72">
+        <v>8</v>
+      </c>
+      <c r="AE10" s="73"/>
+      <c r="AF10" s="48">
+        <v>10</v>
+      </c>
+      <c r="AG10" s="73"/>
+      <c r="AH10" s="71">
+        <v>9</v>
+      </c>
+      <c r="AI10" s="49"/>
+      <c r="AL10" s="24"/>
+      <c r="AM10" s="44"/>
+      <c r="AN10" s="24"/>
+      <c r="AO10" s="24"/>
+      <c r="AP10" s="24"/>
+      <c r="AQ10" s="24"/>
+      <c r="AR10" s="24"/>
+      <c r="AS10" s="24"/>
+      <c r="BH10" s="70">
+        <v>6</v>
+      </c>
+      <c r="BI10" s="44"/>
+      <c r="BJ10" s="50"/>
+      <c r="BK10" s="52"/>
+      <c r="BL10" s="24"/>
+      <c r="BM10" s="24"/>
     </row>
-    <row r="11" spans="2:47" ht="15" customHeight="1">
+    <row r="11" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C11" s="1"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="11">
+      <c r="F11" s="10">
         <v>8</v>
       </c>
-      <c r="G11" s="2"/>
-      <c r="H11" s="2"/>
-      <c r="I11" s="14">
+      <c r="I11" s="13">
         <v>9</v>
       </c>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="17"/>
-      <c r="N11" s="42">
+      <c r="M11" s="16"/>
+      <c r="N11" s="20">
         <v>7</v>
       </c>
-      <c r="O11" s="43"/>
-      <c r="P11" s="42">
+      <c r="O11" s="21"/>
+      <c r="P11" s="20">
         <v>2</v>
       </c>
-      <c r="Q11" s="43"/>
-      <c r="R11" s="42">
+      <c r="Q11" s="21"/>
+      <c r="R11" s="20">
         <v>2</v>
       </c>
-      <c r="S11" s="44"/>
-      <c r="T11" s="55">
+      <c r="S11" s="28"/>
+      <c r="T11" s="40">
         <v>2</v>
       </c>
-      <c r="U11" s="43"/>
-      <c r="V11" s="42">
+      <c r="U11" s="21"/>
+      <c r="V11" s="20">
         <v>2</v>
       </c>
-      <c r="W11" s="43"/>
-      <c r="X11" s="25">
+      <c r="W11" s="21"/>
+      <c r="X11" s="43">
         <v>1</v>
       </c>
-      <c r="Y11" s="24"/>
-      <c r="AB11" s="23">
+      <c r="Y11" s="44"/>
+      <c r="AA11" s="74"/>
+      <c r="AB11" s="53" t="s">
+        <v>12</v>
+      </c>
+      <c r="AC11" s="54"/>
+      <c r="AD11" s="54"/>
+      <c r="AE11" s="54"/>
+      <c r="AF11" s="54"/>
+      <c r="AG11" s="54"/>
+      <c r="AH11" s="54"/>
+      <c r="AI11" s="55"/>
+      <c r="AL11" s="24"/>
+      <c r="AM11" s="44"/>
+      <c r="AN11" s="24"/>
+      <c r="AO11" s="24"/>
+      <c r="AP11" s="24"/>
+      <c r="AQ11" s="24"/>
+      <c r="AR11" s="24"/>
+      <c r="AS11" s="24"/>
+      <c r="BH11" s="70">
         <v>7</v>
       </c>
-      <c r="AC11" s="24"/>
-      <c r="AD11" s="22"/>
-      <c r="AE11" s="22"/>
-      <c r="AF11" s="22"/>
-      <c r="AG11" s="22"/>
-      <c r="AH11" s="22"/>
-      <c r="AI11" s="22"/>
-      <c r="AQ11" s="11"/>
-      <c r="AR11" s="2"/>
-      <c r="AS11" s="2"/>
-      <c r="AT11" s="13"/>
+      <c r="BI11" s="44"/>
+      <c r="BJ11" s="50"/>
+      <c r="BK11" s="52"/>
+      <c r="BL11" s="24"/>
+      <c r="BM11" s="24"/>
     </row>
-    <row r="12" spans="2:47" ht="15" customHeight="1">
+    <row r="12" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C12" s="1"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="8"/>
-      <c r="I12" s="2"/>
-      <c r="J12" s="2"/>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="17"/>
-      <c r="N12" s="42">
+      <c r="G12" s="8"/>
+      <c r="H12" s="7"/>
+      <c r="M12" s="16"/>
+      <c r="N12" s="20">
         <v>8</v>
       </c>
-      <c r="O12" s="43"/>
-      <c r="P12" s="42">
+      <c r="O12" s="21"/>
+      <c r="P12" s="20">
         <v>-1</v>
       </c>
-      <c r="Q12" s="43"/>
-      <c r="R12" s="42">
+      <c r="Q12" s="21"/>
+      <c r="R12" s="20">
         <v>-3</v>
       </c>
-      <c r="S12" s="44"/>
-      <c r="T12" s="55">
+      <c r="S12" s="28"/>
+      <c r="T12" s="40">
         <v>-1</v>
       </c>
-      <c r="U12" s="43"/>
-      <c r="V12" s="42">
+      <c r="U12" s="21"/>
+      <c r="V12" s="20">
         <v>-3</v>
       </c>
-      <c r="W12" s="43"/>
-      <c r="X12" s="25">
+      <c r="W12" s="21"/>
+      <c r="X12" s="43">
         <v>1</v>
       </c>
-      <c r="Y12" s="24"/>
-      <c r="AB12" s="23">
+      <c r="Y12" s="44"/>
+      <c r="AA12" s="74"/>
+      <c r="AB12" s="50">
+        <v>7</v>
+      </c>
+      <c r="AC12" s="44"/>
+      <c r="AD12" s="79">
+        <v>11</v>
+      </c>
+      <c r="AE12" s="56"/>
+      <c r="AF12" s="38">
+        <v>15</v>
+      </c>
+      <c r="AG12" s="56"/>
+      <c r="AH12" s="70">
+        <v>13</v>
+      </c>
+      <c r="AI12" s="44"/>
+      <c r="AL12" s="24"/>
+      <c r="AM12" s="44"/>
+      <c r="AN12" s="24"/>
+      <c r="AO12" s="24"/>
+      <c r="AP12" s="24"/>
+      <c r="AQ12" s="24"/>
+      <c r="AR12" s="24"/>
+      <c r="AS12" s="24"/>
+      <c r="BH12" s="70">
         <v>8</v>
       </c>
-      <c r="AC12" s="24"/>
-      <c r="AD12" s="22"/>
-      <c r="AE12" s="22"/>
-      <c r="AF12" s="22"/>
-      <c r="AG12" s="22"/>
-      <c r="AH12" s="22"/>
-      <c r="AI12" s="22"/>
-      <c r="AQ12" s="2"/>
-      <c r="AR12" s="9"/>
-      <c r="AS12" s="8"/>
+      <c r="BI12" s="44"/>
+      <c r="BJ12" s="50"/>
+      <c r="BK12" s="52"/>
+      <c r="BL12" s="24"/>
+      <c r="BM12" s="24"/>
     </row>
-    <row r="13" spans="2:47" ht="15" customHeight="1">
+    <row r="13" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="23">
+      <c r="G13" s="24">
         <v>10</v>
       </c>
-      <c r="H13" s="23"/>
-      <c r="I13" s="2"/>
-      <c r="J13" s="2"/>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="17"/>
-      <c r="N13" s="42">
+      <c r="H13" s="24"/>
+      <c r="M13" s="16"/>
+      <c r="N13" s="20">
         <v>9</v>
       </c>
-      <c r="O13" s="43"/>
-      <c r="P13" s="42">
+      <c r="O13" s="21"/>
+      <c r="P13" s="20">
         <v>1</v>
       </c>
-      <c r="Q13" s="43"/>
-      <c r="R13" s="42">
+      <c r="Q13" s="21"/>
+      <c r="R13" s="20">
         <v>-3</v>
       </c>
-      <c r="S13" s="44"/>
-      <c r="T13" s="55">
+      <c r="S13" s="28"/>
+      <c r="T13" s="40">
         <v>1</v>
       </c>
-      <c r="U13" s="43"/>
-      <c r="V13" s="42">
+      <c r="U13" s="21"/>
+      <c r="V13" s="20">
         <v>-3</v>
       </c>
-      <c r="W13" s="43"/>
-      <c r="X13" s="25">
+      <c r="W13" s="21"/>
+      <c r="X13" s="43">
         <v>1</v>
       </c>
-      <c r="Y13" s="24"/>
-      <c r="AB13" s="23">
+      <c r="Y13" s="44"/>
+      <c r="AA13" s="74"/>
+      <c r="AB13" s="50">
+        <v>8</v>
+      </c>
+      <c r="AC13" s="44"/>
+      <c r="AD13" s="50">
+        <v>12</v>
+      </c>
+      <c r="AE13" s="52"/>
+      <c r="AF13" s="43">
+        <v>15</v>
+      </c>
+      <c r="AG13" s="52"/>
+      <c r="AH13" s="70">
+        <v>11</v>
+      </c>
+      <c r="AI13" s="44"/>
+      <c r="AL13" s="24"/>
+      <c r="AM13" s="44"/>
+      <c r="AN13" s="24"/>
+      <c r="AO13" s="24"/>
+      <c r="AP13" s="24"/>
+      <c r="AQ13" s="24"/>
+      <c r="AR13" s="24"/>
+      <c r="AS13" s="24"/>
+      <c r="BH13" s="70">
         <v>9</v>
       </c>
-      <c r="AC13" s="24"/>
-      <c r="AD13" s="22"/>
-      <c r="AE13" s="22"/>
-      <c r="AF13" s="22"/>
-      <c r="AG13" s="22"/>
-      <c r="AH13" s="22"/>
-      <c r="AI13" s="22"/>
+      <c r="BI13" s="44"/>
+      <c r="BJ13" s="50"/>
+      <c r="BK13" s="52"/>
+      <c r="BL13" s="24"/>
+      <c r="BM13" s="24"/>
     </row>
-    <row r="14" spans="2:47" ht="15" customHeight="1">
-      <c r="C14" s="5"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="6"/>
-      <c r="M14" s="19"/>
-      <c r="N14" s="45">
+    <row r="14" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C14" s="4"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5"/>
+      <c r="G14" s="5"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
+      <c r="J14" s="5"/>
+      <c r="K14" s="5"/>
+      <c r="L14" s="5"/>
+      <c r="M14" s="18"/>
+      <c r="N14" s="22">
         <v>10</v>
       </c>
-      <c r="O14" s="46"/>
-      <c r="P14" s="45">
+      <c r="O14" s="23"/>
+      <c r="P14" s="22">
         <v>0</v>
       </c>
-      <c r="Q14" s="46"/>
-      <c r="R14" s="45">
+      <c r="Q14" s="23"/>
+      <c r="R14" s="22">
         <v>-4</v>
       </c>
-      <c r="S14" s="47"/>
-      <c r="T14" s="50">
+      <c r="S14" s="29"/>
+      <c r="T14" s="45">
         <v>0</v>
       </c>
-      <c r="U14" s="51"/>
-      <c r="V14" s="52">
+      <c r="U14" s="46"/>
+      <c r="V14" s="47">
         <v>-4</v>
       </c>
-      <c r="W14" s="51"/>
-      <c r="X14" s="53">
+      <c r="W14" s="46"/>
+      <c r="X14" s="48">
         <v>1</v>
       </c>
-      <c r="Y14" s="54"/>
-      <c r="AB14" s="23">
+      <c r="Y14" s="49"/>
+      <c r="AA14" s="74"/>
+      <c r="AB14" s="50">
+        <v>9</v>
+      </c>
+      <c r="AC14" s="44"/>
+      <c r="AD14" s="50">
+        <v>12</v>
+      </c>
+      <c r="AE14" s="52"/>
+      <c r="AF14" s="43">
+        <v>18</v>
+      </c>
+      <c r="AG14" s="52"/>
+      <c r="AH14" s="70">
+        <v>15</v>
+      </c>
+      <c r="AI14" s="44"/>
+      <c r="AL14" s="24"/>
+      <c r="AM14" s="44"/>
+      <c r="AN14" s="24"/>
+      <c r="AO14" s="24"/>
+      <c r="AP14" s="24"/>
+      <c r="AQ14" s="24"/>
+      <c r="AR14" s="24"/>
+      <c r="AS14" s="24"/>
+      <c r="BH14" s="70">
         <v>10</v>
       </c>
-      <c r="AC14" s="24"/>
-      <c r="AD14" s="22"/>
-      <c r="AE14" s="22"/>
-      <c r="AF14" s="22"/>
-      <c r="AG14" s="22"/>
-      <c r="AH14" s="22"/>
-      <c r="AI14" s="22"/>
+      <c r="BI14" s="44"/>
+      <c r="BJ14" s="50"/>
+      <c r="BK14" s="52"/>
+      <c r="BL14" s="24"/>
+      <c r="BM14" s="24"/>
     </row>
-    <row r="15" spans="2:47" ht="15" customHeight="1">
-      <c r="C15" s="3"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4"/>
-      <c r="K15" s="4"/>
-      <c r="L15" s="4"/>
-      <c r="M15" s="18"/>
-      <c r="N15" s="34" t="s">
+    <row r="15" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C15" s="2"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
+      <c r="J15" s="3"/>
+      <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="17"/>
+      <c r="N15" s="57" t="s">
         <v>6</v>
       </c>
-      <c r="O15" s="35"/>
-      <c r="P15" s="35"/>
-      <c r="Q15" s="35"/>
-      <c r="R15" s="35"/>
-      <c r="S15" s="36"/>
-      <c r="T15" s="31"/>
-      <c r="U15" s="32"/>
-      <c r="V15" s="32"/>
-      <c r="W15" s="32"/>
-      <c r="X15" s="32"/>
-      <c r="Y15" s="33"/>
-      <c r="AB15" s="22"/>
-      <c r="AC15" s="22"/>
-      <c r="AD15" s="22"/>
-      <c r="AE15" s="22"/>
-      <c r="AF15" s="22"/>
-      <c r="AG15" s="22"/>
-      <c r="AH15" s="22"/>
-      <c r="AI15" s="22"/>
+      <c r="O15" s="58"/>
+      <c r="P15" s="58"/>
+      <c r="Q15" s="58"/>
+      <c r="R15" s="58"/>
+      <c r="S15" s="59"/>
+      <c r="T15" s="53"/>
+      <c r="U15" s="54"/>
+      <c r="V15" s="54"/>
+      <c r="W15" s="54"/>
+      <c r="X15" s="54"/>
+      <c r="Y15" s="55"/>
+      <c r="AA15" s="74"/>
+      <c r="AB15" s="50">
+        <v>10</v>
+      </c>
+      <c r="AC15" s="44"/>
+      <c r="AD15" s="50">
+        <v>12</v>
+      </c>
+      <c r="AE15" s="52"/>
+      <c r="AF15" s="43">
+        <v>14</v>
+      </c>
+      <c r="AG15" s="52"/>
+      <c r="AH15" s="70">
+        <v>18</v>
+      </c>
+      <c r="AI15" s="44"/>
+      <c r="AZ15" s="63"/>
+      <c r="BA15" s="63"/>
+      <c r="BH15" s="70">
+        <v>11</v>
+      </c>
+      <c r="BI15" s="44"/>
+      <c r="BJ15" s="50"/>
+      <c r="BK15" s="52"/>
+      <c r="BL15" s="24"/>
+      <c r="BM15" s="24"/>
     </row>
-    <row r="16" spans="2:47" ht="15" customHeight="1">
+    <row r="16" spans="3:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C16" s="1"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
-      <c r="H16" s="2"/>
-      <c r="I16" s="2"/>
-      <c r="J16" s="2"/>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="17"/>
-      <c r="N16" s="48"/>
-      <c r="O16" s="49"/>
-      <c r="P16" s="39" t="s">
+      <c r="M16" s="16"/>
+      <c r="N16" s="41"/>
+      <c r="O16" s="42"/>
+      <c r="P16" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="Q16" s="38"/>
-      <c r="R16" s="39" t="s">
+      <c r="Q16" s="26"/>
+      <c r="R16" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="S16" s="41"/>
-      <c r="T16" s="37" t="s">
+      <c r="S16" s="27"/>
+      <c r="T16" s="33" t="s">
         <v>0</v>
       </c>
-      <c r="U16" s="38"/>
-      <c r="V16" s="39" t="s">
+      <c r="U16" s="26"/>
+      <c r="V16" s="25" t="s">
         <v>1</v>
       </c>
-      <c r="W16" s="40"/>
-      <c r="X16" s="39" t="s">
+      <c r="W16" s="34"/>
+      <c r="X16" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="Y16" s="41"/>
-      <c r="AB16" s="23"/>
-      <c r="AC16" s="24"/>
-      <c r="AD16" s="22"/>
-      <c r="AE16" s="22"/>
-      <c r="AF16" s="22"/>
-      <c r="AG16" s="22"/>
-      <c r="AH16" s="22"/>
-      <c r="AI16" s="22"/>
+      <c r="Y16" s="27"/>
+      <c r="AA16" s="74"/>
+      <c r="AB16" s="50">
+        <v>11</v>
+      </c>
+      <c r="AC16" s="44"/>
+      <c r="AD16" s="50">
+        <v>17</v>
+      </c>
+      <c r="AE16" s="52"/>
+      <c r="AF16" s="43">
+        <v>20</v>
+      </c>
+      <c r="AG16" s="52"/>
+      <c r="AH16" s="70">
+        <v>16</v>
+      </c>
+      <c r="AI16" s="44"/>
+      <c r="AZ16" s="63"/>
+      <c r="BA16" s="63"/>
+      <c r="BH16" s="70">
+        <v>12</v>
+      </c>
+      <c r="BI16" s="44"/>
+      <c r="BJ16" s="50"/>
+      <c r="BK16" s="52"/>
+      <c r="BL16" s="24"/>
+      <c r="BM16" s="24"/>
     </row>
-    <row r="17" spans="3:35" ht="15" customHeight="1" thickBot="1">
+    <row r="17" spans="2:65" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C17" s="1"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
-      <c r="I17" s="7"/>
-      <c r="J17" s="15"/>
-      <c r="K17" s="2"/>
-      <c r="L17" s="2"/>
-      <c r="M17" s="17"/>
-      <c r="N17" s="42">
+      <c r="E17" s="19">
+        <v>12</v>
+      </c>
+      <c r="F17" s="6"/>
+      <c r="G17" s="6"/>
+      <c r="H17" s="6"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="64">
         <v>11</v>
       </c>
-      <c r="O17" s="43"/>
-      <c r="P17" s="42"/>
-      <c r="Q17" s="43"/>
-      <c r="R17" s="42"/>
-      <c r="S17" s="44"/>
-      <c r="T17" s="21"/>
-      <c r="U17" s="22"/>
-      <c r="V17" s="22"/>
-      <c r="W17" s="22"/>
-      <c r="X17" s="29"/>
-      <c r="Y17" s="30"/>
-      <c r="AB17" s="23"/>
-      <c r="AC17" s="24"/>
-      <c r="AD17" s="22"/>
-      <c r="AE17" s="22"/>
-      <c r="AF17" s="22"/>
-      <c r="AG17" s="22"/>
-      <c r="AH17" s="22"/>
-      <c r="AI17" s="22"/>
+      <c r="M17" s="16"/>
+      <c r="N17" s="20">
+        <v>11</v>
+      </c>
+      <c r="O17" s="21"/>
+      <c r="P17" s="20">
+        <v>-2</v>
+      </c>
+      <c r="Q17" s="21"/>
+      <c r="R17" s="20">
+        <v>4</v>
+      </c>
+      <c r="S17" s="28"/>
+      <c r="T17" s="79">
+        <v>-2</v>
+      </c>
+      <c r="U17" s="56"/>
+      <c r="V17" s="38">
+        <v>4</v>
+      </c>
+      <c r="W17" s="56"/>
+      <c r="X17" s="51">
+        <v>-1</v>
+      </c>
+      <c r="Y17" s="39"/>
+      <c r="AA17" s="74"/>
+      <c r="AB17" s="50">
+        <v>12</v>
+      </c>
+      <c r="AC17" s="44"/>
+      <c r="AD17" s="50">
+        <v>16</v>
+      </c>
+      <c r="AE17" s="52"/>
+      <c r="AF17" s="43">
+        <v>20</v>
+      </c>
+      <c r="AG17" s="52"/>
+      <c r="AH17" s="70">
+        <v>19</v>
+      </c>
+      <c r="AI17" s="44"/>
+      <c r="AZ17" s="63"/>
+      <c r="BA17" s="63"/>
+      <c r="BH17" s="70">
+        <v>13</v>
+      </c>
+      <c r="BI17" s="44"/>
+      <c r="BJ17" s="50"/>
+      <c r="BK17" s="52"/>
+      <c r="BL17" s="24"/>
+      <c r="BM17" s="24"/>
     </row>
-    <row r="18" spans="3:35" ht="15" customHeight="1">
+    <row r="18" spans="2:65" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C18" s="1"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-      <c r="H18" s="2"/>
-      <c r="I18" s="2"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="2"/>
-      <c r="M18" s="17"/>
-      <c r="N18" s="42">
+      <c r="D18" s="19">
+        <v>14</v>
+      </c>
+      <c r="E18" s="7"/>
+      <c r="J18" s="8"/>
+      <c r="K18" s="64">
+        <v>13</v>
+      </c>
+      <c r="M18" s="16"/>
+      <c r="N18" s="20">
         <v>12</v>
       </c>
-      <c r="O18" s="43"/>
-      <c r="P18" s="42"/>
-      <c r="Q18" s="43"/>
-      <c r="R18" s="42"/>
-      <c r="S18" s="44"/>
-      <c r="T18" s="21"/>
-      <c r="U18" s="22"/>
-      <c r="V18" s="22"/>
-      <c r="W18" s="22"/>
-      <c r="X18" s="23"/>
-      <c r="Y18" s="24"/>
-      <c r="AB18" s="23"/>
-      <c r="AC18" s="24"/>
-      <c r="AD18" s="22"/>
-      <c r="AE18" s="22"/>
-      <c r="AF18" s="22"/>
-      <c r="AG18" s="22"/>
-      <c r="AH18" s="22"/>
-      <c r="AI18" s="22"/>
+      <c r="O18" s="21"/>
+      <c r="P18" s="20">
+        <v>2</v>
+      </c>
+      <c r="Q18" s="21"/>
+      <c r="R18" s="20">
+        <v>4</v>
+      </c>
+      <c r="S18" s="28"/>
+      <c r="T18" s="50">
+        <v>2</v>
+      </c>
+      <c r="U18" s="52"/>
+      <c r="V18" s="43">
+        <v>4</v>
+      </c>
+      <c r="W18" s="52"/>
+      <c r="X18" s="24">
+        <v>-1</v>
+      </c>
+      <c r="Y18" s="44"/>
+      <c r="AA18" s="74"/>
+      <c r="AB18" s="50">
+        <v>13</v>
+      </c>
+      <c r="AC18" s="44"/>
+      <c r="AD18" s="72">
+        <v>20</v>
+      </c>
+      <c r="AE18" s="73"/>
+      <c r="AF18" s="48">
+        <v>21</v>
+      </c>
+      <c r="AG18" s="73"/>
+      <c r="AH18" s="70">
+        <v>19</v>
+      </c>
+      <c r="AI18" s="44"/>
+      <c r="AJ18" s="63"/>
+      <c r="AZ18" s="63"/>
+      <c r="BA18" s="63"/>
+      <c r="BH18" s="70">
+        <v>14</v>
+      </c>
+      <c r="BI18" s="44"/>
+      <c r="BJ18" s="50"/>
+      <c r="BK18" s="52"/>
+      <c r="BL18" s="24"/>
+      <c r="BM18" s="24"/>
     </row>
-    <row r="19" spans="3:35" ht="15" customHeight="1" thickBot="1">
+    <row r="19" spans="2:65" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C19" s="1"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="2"/>
-      <c r="H19" s="2"/>
-      <c r="I19" s="16"/>
-      <c r="J19" s="8"/>
-      <c r="K19" s="2"/>
-      <c r="L19" s="2"/>
-      <c r="M19" s="17"/>
-      <c r="N19" s="42">
+      <c r="E19" s="8"/>
+      <c r="F19" s="66">
+        <v>17</v>
+      </c>
+      <c r="I19" s="65">
+        <v>16</v>
+      </c>
+      <c r="J19" s="7"/>
+      <c r="M19" s="16"/>
+      <c r="N19" s="20">
         <v>13</v>
       </c>
-      <c r="O19" s="43"/>
-      <c r="P19" s="42"/>
-      <c r="Q19" s="43"/>
-      <c r="R19" s="42"/>
-      <c r="S19" s="44"/>
-      <c r="T19" s="21"/>
-      <c r="U19" s="22"/>
-      <c r="V19" s="22"/>
-      <c r="W19" s="22"/>
-      <c r="X19" s="23"/>
-      <c r="Y19" s="24"/>
-      <c r="AB19" s="23"/>
-      <c r="AC19" s="24"/>
-      <c r="AD19" s="22"/>
-      <c r="AE19" s="22"/>
-      <c r="AF19" s="22"/>
-      <c r="AG19" s="22"/>
-      <c r="AH19" s="22"/>
-      <c r="AI19" s="22"/>
+      <c r="O19" s="21"/>
+      <c r="P19" s="20">
+        <v>-3</v>
+      </c>
+      <c r="Q19" s="21"/>
+      <c r="R19" s="20">
+        <v>3</v>
+      </c>
+      <c r="S19" s="28"/>
+      <c r="T19" s="50">
+        <v>-3</v>
+      </c>
+      <c r="U19" s="52"/>
+      <c r="V19" s="43">
+        <v>3</v>
+      </c>
+      <c r="W19" s="52"/>
+      <c r="X19" s="24">
+        <v>-1</v>
+      </c>
+      <c r="Y19" s="44"/>
+      <c r="AB19" s="53" t="s">
+        <v>13</v>
+      </c>
+      <c r="AC19" s="54"/>
+      <c r="AD19" s="54"/>
+      <c r="AE19" s="54"/>
+      <c r="AF19" s="54"/>
+      <c r="AG19" s="54"/>
+      <c r="AH19" s="54"/>
+      <c r="AI19" s="55"/>
+      <c r="AQ19" s="11"/>
+      <c r="AR19" s="82"/>
+      <c r="AS19" s="82"/>
+      <c r="AT19" s="82"/>
+      <c r="AU19" s="82"/>
+      <c r="AV19" s="9"/>
+      <c r="AZ19" s="63"/>
+      <c r="BA19" s="63"/>
+      <c r="BH19" s="70">
+        <v>15</v>
+      </c>
+      <c r="BI19" s="44"/>
+      <c r="BJ19" s="50"/>
+      <c r="BK19" s="52"/>
+      <c r="BL19" s="24"/>
+      <c r="BM19" s="24"/>
     </row>
-    <row r="20" spans="3:35" ht="15" customHeight="1">
+    <row r="20" spans="2:65" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="C20" s="1"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="2"/>
-      <c r="H20" s="2"/>
-      <c r="I20" s="12"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="2"/>
-      <c r="L20" s="2"/>
-      <c r="M20" s="17"/>
-      <c r="N20" s="42">
+      <c r="E20" s="19">
+        <v>18</v>
+      </c>
+      <c r="F20" s="9"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="64">
+        <v>15</v>
+      </c>
+      <c r="M20" s="16"/>
+      <c r="N20" s="20">
         <v>14</v>
       </c>
-      <c r="O20" s="43"/>
-      <c r="P20" s="42"/>
-      <c r="Q20" s="43"/>
-      <c r="R20" s="42"/>
-      <c r="S20" s="44"/>
-      <c r="T20" s="21"/>
-      <c r="U20" s="22"/>
-      <c r="V20" s="22"/>
-      <c r="W20" s="22"/>
-      <c r="X20" s="23"/>
-      <c r="Y20" s="24"/>
-      <c r="AB20" s="23"/>
-      <c r="AC20" s="24"/>
-      <c r="AD20" s="22"/>
-      <c r="AE20" s="22"/>
-      <c r="AF20" s="22"/>
-      <c r="AG20" s="22"/>
-      <c r="AH20" s="22"/>
-      <c r="AI20" s="22"/>
+      <c r="O20" s="21"/>
+      <c r="P20" s="20">
+        <v>3</v>
+      </c>
+      <c r="Q20" s="21"/>
+      <c r="R20" s="20">
+        <v>3</v>
+      </c>
+      <c r="S20" s="28"/>
+      <c r="T20" s="50">
+        <v>3</v>
+      </c>
+      <c r="U20" s="52"/>
+      <c r="V20" s="43">
+        <v>3</v>
+      </c>
+      <c r="W20" s="52"/>
+      <c r="X20" s="24">
+        <v>-1</v>
+      </c>
+      <c r="Y20" s="44"/>
+      <c r="AB20" s="24"/>
+      <c r="AC20" s="44"/>
+      <c r="AD20" s="24"/>
+      <c r="AE20" s="24"/>
+      <c r="AF20" s="24"/>
+      <c r="AG20" s="24"/>
+      <c r="AH20" s="24"/>
+      <c r="AI20" s="24"/>
+      <c r="AQ20" s="80"/>
+      <c r="AR20" s="6"/>
+      <c r="AS20" s="6"/>
+      <c r="AT20" s="6"/>
+      <c r="AU20" s="6"/>
+      <c r="AV20" s="81"/>
+      <c r="AZ20" s="63"/>
+      <c r="BA20" s="63"/>
+      <c r="BH20" s="70">
+        <v>16</v>
+      </c>
+      <c r="BI20" s="44"/>
+      <c r="BJ20" s="50"/>
+      <c r="BK20" s="52"/>
+      <c r="BL20" s="24"/>
+      <c r="BM20" s="24"/>
     </row>
-    <row r="21" spans="3:35" ht="15" customHeight="1">
+    <row r="21" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C21" s="1"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
-      <c r="F21" s="11"/>
-      <c r="G21" s="2"/>
-      <c r="H21" s="2"/>
-      <c r="I21" s="13"/>
-      <c r="J21" s="2"/>
-      <c r="K21" s="2"/>
-      <c r="L21" s="2"/>
-      <c r="M21" s="17"/>
-      <c r="N21" s="42">
+      <c r="F21" s="10"/>
+      <c r="I21" s="12"/>
+      <c r="M21" s="16"/>
+      <c r="N21" s="20">
         <v>15</v>
       </c>
-      <c r="O21" s="43"/>
-      <c r="P21" s="42"/>
-      <c r="Q21" s="43"/>
-      <c r="R21" s="42"/>
-      <c r="S21" s="44"/>
-      <c r="T21" s="21"/>
-      <c r="U21" s="22"/>
-      <c r="V21" s="22"/>
-      <c r="W21" s="22"/>
-      <c r="X21" s="23"/>
-      <c r="Y21" s="24"/>
-      <c r="AB21" s="23"/>
-      <c r="AC21" s="24"/>
-      <c r="AD21" s="22"/>
-      <c r="AE21" s="22"/>
-      <c r="AF21" s="22"/>
-      <c r="AG21" s="22"/>
-      <c r="AH21" s="22"/>
-      <c r="AI21" s="22"/>
+      <c r="O21" s="21"/>
+      <c r="P21" s="20">
+        <v>-2</v>
+      </c>
+      <c r="Q21" s="21"/>
+      <c r="R21" s="20">
+        <v>2</v>
+      </c>
+      <c r="S21" s="28"/>
+      <c r="T21" s="50">
+        <v>-2</v>
+      </c>
+      <c r="U21" s="52"/>
+      <c r="V21" s="43">
+        <v>2</v>
+      </c>
+      <c r="W21" s="52"/>
+      <c r="X21" s="24">
+        <v>-1</v>
+      </c>
+      <c r="Y21" s="44"/>
+      <c r="AB21" s="24"/>
+      <c r="AC21" s="44"/>
+      <c r="AD21" s="24"/>
+      <c r="AE21" s="24"/>
+      <c r="AF21" s="24"/>
+      <c r="AG21" s="24"/>
+      <c r="AH21" s="24"/>
+      <c r="AI21" s="24"/>
+      <c r="AZ21" s="63"/>
+      <c r="BA21" s="63"/>
+      <c r="BH21" s="70">
+        <v>17</v>
+      </c>
+      <c r="BI21" s="44"/>
+      <c r="BJ21" s="50"/>
+      <c r="BK21" s="52"/>
+      <c r="BL21" s="24"/>
+      <c r="BM21" s="24"/>
     </row>
-    <row r="22" spans="3:35" ht="15" customHeight="1">
+    <row r="22" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C22" s="1"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="11"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="13"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="17"/>
-      <c r="N22" s="42">
+      <c r="F22" s="10"/>
+      <c r="I22" s="12"/>
+      <c r="M22" s="16"/>
+      <c r="N22" s="20">
         <v>16</v>
       </c>
-      <c r="O22" s="43"/>
-      <c r="P22" s="42"/>
-      <c r="Q22" s="43"/>
-      <c r="R22" s="42"/>
-      <c r="S22" s="44"/>
-      <c r="T22" s="21"/>
-      <c r="U22" s="22"/>
-      <c r="V22" s="22"/>
-      <c r="W22" s="22"/>
-      <c r="X22" s="23"/>
-      <c r="Y22" s="24"/>
-      <c r="AB22" s="23"/>
-      <c r="AC22" s="24"/>
-      <c r="AD22" s="22"/>
-      <c r="AE22" s="22"/>
-      <c r="AF22" s="22"/>
-      <c r="AG22" s="22"/>
-      <c r="AH22" s="22"/>
-      <c r="AI22" s="22"/>
+      <c r="O22" s="21"/>
+      <c r="P22" s="20">
+        <v>-1</v>
+      </c>
+      <c r="Q22" s="21"/>
+      <c r="R22" s="20">
+        <v>2</v>
+      </c>
+      <c r="S22" s="28"/>
+      <c r="T22" s="50">
+        <v>-1</v>
+      </c>
+      <c r="U22" s="52"/>
+      <c r="V22" s="43">
+        <v>2</v>
+      </c>
+      <c r="W22" s="52"/>
+      <c r="X22" s="24">
+        <v>-1</v>
+      </c>
+      <c r="Y22" s="44"/>
+      <c r="AB22" s="24"/>
+      <c r="AC22" s="44"/>
+      <c r="AD22" s="24"/>
+      <c r="AE22" s="24"/>
+      <c r="AF22" s="24"/>
+      <c r="AG22" s="24"/>
+      <c r="AH22" s="24"/>
+      <c r="AI22" s="24"/>
+      <c r="AZ22" s="63"/>
+      <c r="BA22" s="63"/>
+      <c r="BH22" s="70">
+        <v>18</v>
+      </c>
+      <c r="BI22" s="44"/>
+      <c r="BJ22" s="50"/>
+      <c r="BK22" s="52"/>
+      <c r="BL22" s="24"/>
+      <c r="BM22" s="24"/>
     </row>
-    <row r="23" spans="3:35" ht="15" customHeight="1">
+    <row r="23" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C23" s="1"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-      <c r="F23" s="11"/>
-      <c r="G23" s="2"/>
-      <c r="H23" s="2"/>
-      <c r="I23" s="13"/>
-      <c r="J23" s="2"/>
-      <c r="K23" s="2"/>
-      <c r="L23" s="2"/>
-      <c r="M23" s="17"/>
-      <c r="N23" s="42">
+      <c r="F23" s="10"/>
+      <c r="I23" s="12"/>
+      <c r="M23" s="16"/>
+      <c r="N23" s="20">
         <v>17</v>
       </c>
-      <c r="O23" s="43"/>
-      <c r="P23" s="42"/>
-      <c r="Q23" s="43"/>
-      <c r="R23" s="42"/>
-      <c r="S23" s="44"/>
-      <c r="T23" s="21"/>
-      <c r="U23" s="22"/>
-      <c r="V23" s="22"/>
-      <c r="W23" s="22"/>
-      <c r="X23" s="23"/>
-      <c r="Y23" s="24"/>
-      <c r="AB23" s="23"/>
-      <c r="AC23" s="24"/>
-      <c r="AD23" s="22"/>
-      <c r="AE23" s="22"/>
-      <c r="AF23" s="22"/>
-      <c r="AG23" s="22"/>
-      <c r="AH23" s="22"/>
-      <c r="AI23" s="22"/>
+      <c r="O23" s="21"/>
+      <c r="P23" s="20">
+        <v>1</v>
+      </c>
+      <c r="Q23" s="21"/>
+      <c r="R23" s="20">
+        <v>2</v>
+      </c>
+      <c r="S23" s="28"/>
+      <c r="T23" s="50">
+        <v>1</v>
+      </c>
+      <c r="U23" s="52"/>
+      <c r="V23" s="43">
+        <v>2</v>
+      </c>
+      <c r="W23" s="52"/>
+      <c r="X23" s="24">
+        <v>-1</v>
+      </c>
+      <c r="Y23" s="44"/>
+      <c r="AB23" s="24"/>
+      <c r="AC23" s="44"/>
+      <c r="AD23" s="24"/>
+      <c r="AE23" s="24"/>
+      <c r="AF23" s="24"/>
+      <c r="AG23" s="24"/>
+      <c r="AH23" s="24"/>
+      <c r="AI23" s="24"/>
+      <c r="BH23" s="70">
+        <v>19</v>
+      </c>
+      <c r="BI23" s="44"/>
+      <c r="BJ23" s="50"/>
+      <c r="BK23" s="52"/>
+      <c r="BL23" s="24"/>
+      <c r="BM23" s="24"/>
     </row>
-    <row r="24" spans="3:35" ht="15" customHeight="1">
+    <row r="24" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C24" s="1"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="11"/>
-      <c r="G24" s="2"/>
-      <c r="H24" s="2"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="2"/>
-      <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="17"/>
-      <c r="N24" s="42">
+      <c r="F24" s="67">
+        <v>20</v>
+      </c>
+      <c r="I24" s="68">
+        <v>19</v>
+      </c>
+      <c r="M24" s="16"/>
+      <c r="N24" s="20">
         <v>18</v>
       </c>
-      <c r="O24" s="43"/>
-      <c r="P24" s="42"/>
-      <c r="Q24" s="43"/>
-      <c r="R24" s="42"/>
-      <c r="S24" s="44"/>
-      <c r="T24" s="21"/>
-      <c r="U24" s="22"/>
-      <c r="V24" s="22"/>
-      <c r="W24" s="22"/>
-      <c r="X24" s="23"/>
-      <c r="Y24" s="24"/>
-      <c r="AB24" s="23"/>
-      <c r="AC24" s="24"/>
-      <c r="AD24" s="22"/>
-      <c r="AE24" s="22"/>
-      <c r="AF24" s="22"/>
-      <c r="AG24" s="22"/>
-      <c r="AH24" s="22"/>
-      <c r="AI24" s="22"/>
+      <c r="O24" s="21"/>
+      <c r="P24" s="20">
+        <v>2</v>
+      </c>
+      <c r="Q24" s="21"/>
+      <c r="R24" s="20">
+        <v>2</v>
+      </c>
+      <c r="S24" s="28"/>
+      <c r="T24" s="50">
+        <v>2</v>
+      </c>
+      <c r="U24" s="52"/>
+      <c r="V24" s="43">
+        <v>2</v>
+      </c>
+      <c r="W24" s="52"/>
+      <c r="X24" s="24">
+        <v>-1</v>
+      </c>
+      <c r="Y24" s="44"/>
+      <c r="AB24" s="24"/>
+      <c r="AC24" s="44"/>
+      <c r="AD24" s="24"/>
+      <c r="AE24" s="24"/>
+      <c r="AF24" s="24"/>
+      <c r="AG24" s="24"/>
+      <c r="AH24" s="24"/>
+      <c r="AI24" s="24"/>
+      <c r="BH24" s="70">
+        <v>20</v>
+      </c>
+      <c r="BI24" s="44"/>
+      <c r="BJ24" s="50"/>
+      <c r="BK24" s="52"/>
+      <c r="BL24" s="24"/>
+      <c r="BM24" s="24"/>
     </row>
-    <row r="25" spans="3:35" ht="15" customHeight="1">
+    <row r="25" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C25" s="1"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-      <c r="F25" s="2"/>
-      <c r="G25" s="9"/>
-      <c r="H25" s="8"/>
-      <c r="I25" s="2"/>
-      <c r="J25" s="2"/>
-      <c r="K25" s="2"/>
-      <c r="L25" s="2"/>
-      <c r="M25" s="17"/>
-      <c r="N25" s="42">
+      <c r="G25" s="8"/>
+      <c r="H25" s="7"/>
+      <c r="M25" s="16"/>
+      <c r="N25" s="20">
         <v>19</v>
       </c>
-      <c r="O25" s="43"/>
-      <c r="P25" s="42"/>
-      <c r="Q25" s="43"/>
-      <c r="R25" s="42"/>
-      <c r="S25" s="44"/>
-      <c r="T25" s="21"/>
-      <c r="U25" s="22"/>
-      <c r="V25" s="22"/>
-      <c r="W25" s="22"/>
-      <c r="X25" s="23"/>
-      <c r="Y25" s="24"/>
-      <c r="AB25" s="23"/>
-      <c r="AC25" s="24"/>
-      <c r="AD25" s="22"/>
-      <c r="AE25" s="22"/>
-      <c r="AF25" s="22"/>
-      <c r="AG25" s="22"/>
-      <c r="AH25" s="22"/>
-      <c r="AI25" s="22"/>
+      <c r="O25" s="21"/>
+      <c r="P25" s="20">
+        <v>-1</v>
+      </c>
+      <c r="Q25" s="21"/>
+      <c r="R25" s="20">
+        <v>-3</v>
+      </c>
+      <c r="S25" s="28"/>
+      <c r="T25" s="50">
+        <v>-1</v>
+      </c>
+      <c r="U25" s="52"/>
+      <c r="V25" s="43">
+        <v>-3</v>
+      </c>
+      <c r="W25" s="52"/>
+      <c r="X25" s="24">
+        <v>-1</v>
+      </c>
+      <c r="Y25" s="44"/>
+      <c r="AB25" s="63"/>
+      <c r="AC25" s="63"/>
+      <c r="AD25" s="63"/>
+      <c r="AE25" s="63"/>
+      <c r="AF25" s="63"/>
+      <c r="BH25" s="70">
+        <v>21</v>
+      </c>
+      <c r="BI25" s="44"/>
+      <c r="BJ25" s="50"/>
+      <c r="BK25" s="52"/>
+      <c r="BL25" s="24"/>
+      <c r="BM25" s="24"/>
     </row>
-    <row r="26" spans="3:35" ht="15" customHeight="1">
+    <row r="26" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C26" s="1"/>
-      <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
-      <c r="G26" s="23"/>
-      <c r="H26" s="23"/>
-      <c r="I26" s="2"/>
-      <c r="J26" s="2"/>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
-      <c r="M26" s="17"/>
-      <c r="N26" s="42">
+      <c r="G26" s="69">
+        <v>21</v>
+      </c>
+      <c r="H26" s="69"/>
+      <c r="M26" s="16"/>
+      <c r="N26" s="20">
         <v>20</v>
       </c>
-      <c r="O26" s="43"/>
-      <c r="P26" s="42"/>
-      <c r="Q26" s="43"/>
-      <c r="R26" s="42"/>
-      <c r="S26" s="44"/>
-      <c r="T26" s="21"/>
-      <c r="U26" s="22"/>
-      <c r="V26" s="22"/>
-      <c r="W26" s="22"/>
-      <c r="X26" s="23"/>
-      <c r="Y26" s="24"/>
-      <c r="AB26" s="23"/>
-      <c r="AC26" s="24"/>
-      <c r="AD26" s="22"/>
-      <c r="AE26" s="22"/>
-      <c r="AF26" s="22"/>
-      <c r="AG26" s="22"/>
-      <c r="AH26" s="22"/>
-      <c r="AI26" s="22"/>
+      <c r="O26" s="21"/>
+      <c r="P26" s="20">
+        <v>1</v>
+      </c>
+      <c r="Q26" s="21"/>
+      <c r="R26" s="20">
+        <v>-3</v>
+      </c>
+      <c r="S26" s="28"/>
+      <c r="T26" s="50">
+        <v>1</v>
+      </c>
+      <c r="U26" s="52"/>
+      <c r="V26" s="43">
+        <v>-3</v>
+      </c>
+      <c r="W26" s="52"/>
+      <c r="X26" s="24">
+        <v>-1</v>
+      </c>
+      <c r="Y26" s="44"/>
+      <c r="AB26" s="24"/>
+      <c r="AC26" s="44"/>
+      <c r="AD26" s="24"/>
+      <c r="AE26" s="24"/>
+      <c r="AF26" s="24"/>
+      <c r="AG26" s="24"/>
+      <c r="AH26" s="24"/>
+      <c r="AI26" s="24"/>
+      <c r="BH26" s="70">
+        <v>22</v>
+      </c>
+      <c r="BI26" s="44"/>
+      <c r="BJ26" s="50"/>
+      <c r="BK26" s="52"/>
+      <c r="BL26" s="24"/>
+      <c r="BM26" s="24"/>
     </row>
-    <row r="27" spans="3:35" ht="15" customHeight="1">
-      <c r="C27" s="5"/>
-      <c r="D27" s="6"/>
-      <c r="E27" s="6"/>
-      <c r="F27" s="6"/>
-      <c r="G27" s="6"/>
-      <c r="H27" s="6"/>
-      <c r="I27" s="6"/>
-      <c r="J27" s="6"/>
-      <c r="K27" s="6"/>
-      <c r="L27" s="6"/>
-      <c r="M27" s="19"/>
-      <c r="N27" s="45">
+    <row r="27" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C27" s="4"/>
+      <c r="D27" s="5"/>
+      <c r="E27" s="5"/>
+      <c r="F27" s="5"/>
+      <c r="G27" s="5"/>
+      <c r="H27" s="5"/>
+      <c r="I27" s="5"/>
+      <c r="J27" s="5"/>
+      <c r="K27" s="5"/>
+      <c r="L27" s="5"/>
+      <c r="M27" s="18"/>
+      <c r="N27" s="20">
         <v>21</v>
       </c>
-      <c r="O27" s="46"/>
-      <c r="P27" s="45"/>
-      <c r="Q27" s="46"/>
-      <c r="R27" s="45"/>
-      <c r="S27" s="47"/>
-      <c r="T27" s="21"/>
-      <c r="U27" s="22"/>
-      <c r="V27" s="22"/>
-      <c r="W27" s="22"/>
-      <c r="X27" s="23"/>
-      <c r="Y27" s="24"/>
-      <c r="AB27" s="23"/>
-      <c r="AC27" s="24"/>
-      <c r="AD27" s="22"/>
-      <c r="AE27" s="22"/>
-      <c r="AF27" s="22"/>
-      <c r="AG27" s="22"/>
-      <c r="AH27" s="22"/>
-      <c r="AI27" s="22"/>
+      <c r="O27" s="21"/>
+      <c r="P27" s="20">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="21"/>
+      <c r="R27" s="20">
+        <v>-4</v>
+      </c>
+      <c r="S27" s="28"/>
+      <c r="T27" s="62">
+        <v>0</v>
+      </c>
+      <c r="U27" s="61"/>
+      <c r="V27" s="60">
+        <v>-4</v>
+      </c>
+      <c r="W27" s="61"/>
+      <c r="X27" s="24">
+        <v>-1</v>
+      </c>
+      <c r="Y27" s="44"/>
+      <c r="AB27" s="24"/>
+      <c r="AC27" s="44"/>
+      <c r="AD27" s="24"/>
+      <c r="AE27" s="24"/>
+      <c r="AF27" s="24"/>
+      <c r="AG27" s="24"/>
+      <c r="AH27" s="24"/>
+      <c r="AI27" s="24"/>
+      <c r="BH27" s="70">
+        <v>23</v>
+      </c>
+      <c r="BI27" s="44"/>
+      <c r="BJ27" s="50"/>
+      <c r="BK27" s="52"/>
+      <c r="BL27" s="24"/>
+      <c r="BM27" s="24"/>
     </row>
-    <row r="28" spans="3:35" ht="15" customHeight="1">
-      <c r="N28" s="34" t="s">
-        <v>7</v>
-      </c>
-      <c r="O28" s="35"/>
-      <c r="P28" s="35"/>
-      <c r="Q28" s="35"/>
-      <c r="R28" s="35"/>
-      <c r="S28" s="36"/>
-      <c r="T28" s="31"/>
-      <c r="U28" s="32"/>
-      <c r="V28" s="32"/>
-      <c r="W28" s="32"/>
-      <c r="X28" s="32"/>
-      <c r="Y28" s="33"/>
-      <c r="AB28" s="22"/>
-      <c r="AC28" s="22"/>
-      <c r="AD28" s="22"/>
-      <c r="AE28" s="22"/>
-      <c r="AF28" s="22"/>
-      <c r="AG28" s="22"/>
-      <c r="AH28" s="22"/>
-      <c r="AI28" s="22"/>
+    <row r="28" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B28" s="63"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="3"/>
+      <c r="K28" s="3"/>
+      <c r="L28" s="3"/>
+      <c r="M28" s="3"/>
+      <c r="N28" s="77"/>
+      <c r="O28" s="77"/>
+      <c r="P28" s="77"/>
+      <c r="Q28" s="77"/>
+      <c r="R28" s="77"/>
+      <c r="S28" s="77"/>
+      <c r="T28" s="78"/>
+      <c r="U28" s="78"/>
+      <c r="V28" s="78"/>
+      <c r="W28" s="78"/>
+      <c r="X28" s="78"/>
+      <c r="Y28" s="78"/>
+      <c r="AB28" s="24"/>
+      <c r="AC28" s="24"/>
+      <c r="AD28" s="24"/>
+      <c r="AE28" s="24"/>
+      <c r="AF28" s="24"/>
+      <c r="AG28" s="24"/>
+      <c r="AH28" s="24"/>
+      <c r="AI28" s="24"/>
+      <c r="BH28" s="70">
+        <v>24</v>
+      </c>
+      <c r="BI28" s="44"/>
+      <c r="BJ28" s="50"/>
+      <c r="BK28" s="52"/>
+      <c r="BL28" s="24"/>
+      <c r="BM28" s="24"/>
     </row>
-    <row r="29" spans="3:35" ht="15" customHeight="1">
-      <c r="N29" s="27"/>
-      <c r="O29" s="28"/>
-      <c r="P29" s="29"/>
-      <c r="Q29" s="28"/>
-      <c r="R29" s="29"/>
-      <c r="S29" s="30"/>
-      <c r="T29" s="21"/>
-      <c r="U29" s="22"/>
-      <c r="V29" s="22"/>
-      <c r="W29" s="22"/>
-      <c r="X29" s="23"/>
-      <c r="Y29" s="24"/>
+    <row r="29" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B29" s="63"/>
+      <c r="C29" s="63"/>
+      <c r="D29" s="63"/>
+      <c r="E29" s="63"/>
+      <c r="F29" s="63"/>
+      <c r="G29" s="63"/>
+      <c r="H29" s="63"/>
+      <c r="I29" s="63"/>
+      <c r="J29" s="63"/>
+      <c r="K29" s="63"/>
+      <c r="L29" s="63"/>
+      <c r="M29" s="63"/>
+      <c r="N29" s="76"/>
+      <c r="O29" s="76"/>
+      <c r="P29" s="76"/>
+      <c r="Q29" s="76"/>
+      <c r="R29" s="76"/>
+      <c r="S29" s="76"/>
+      <c r="T29" s="76"/>
+      <c r="U29" s="76"/>
+      <c r="V29" s="76"/>
+      <c r="W29" s="76"/>
+      <c r="X29" s="76"/>
+      <c r="Y29" s="76"/>
+      <c r="Z29" s="63"/>
+      <c r="AB29" s="24"/>
+      <c r="AC29" s="44"/>
+      <c r="AD29" s="24"/>
+      <c r="AE29" s="24"/>
+      <c r="AF29" s="24"/>
+      <c r="AG29" s="24"/>
+      <c r="AH29" s="24"/>
+      <c r="AI29" s="24"/>
+      <c r="BH29" s="70">
+        <v>25</v>
+      </c>
+      <c r="BI29" s="44"/>
+      <c r="BJ29" s="50"/>
+      <c r="BK29" s="52"/>
+      <c r="BL29" s="24"/>
+      <c r="BM29" s="24"/>
     </row>
-    <row r="30" spans="3:35" ht="15" customHeight="1">
-      <c r="N30" s="25"/>
-      <c r="O30" s="26"/>
-      <c r="P30" s="23"/>
-      <c r="Q30" s="26"/>
-      <c r="R30" s="23"/>
-      <c r="S30" s="24"/>
-      <c r="T30" s="21"/>
-      <c r="U30" s="22"/>
-      <c r="V30" s="22"/>
-      <c r="W30" s="22"/>
-      <c r="X30" s="23"/>
-      <c r="Y30" s="24"/>
+    <row r="30" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B30" s="63"/>
+      <c r="C30" s="63"/>
+      <c r="D30" s="63"/>
+      <c r="E30" s="63"/>
+      <c r="F30" s="63"/>
+      <c r="G30" s="63"/>
+      <c r="H30" s="63"/>
+      <c r="I30" s="63"/>
+      <c r="J30" s="63"/>
+      <c r="K30" s="63"/>
+      <c r="L30" s="63"/>
+      <c r="M30" s="63"/>
+      <c r="N30" s="76"/>
+      <c r="O30" s="76"/>
+      <c r="P30" s="76"/>
+      <c r="Q30" s="76"/>
+      <c r="R30" s="76"/>
+      <c r="S30" s="76"/>
+      <c r="T30" s="76"/>
+      <c r="U30" s="76"/>
+      <c r="V30" s="76"/>
+      <c r="W30" s="76"/>
+      <c r="X30" s="76"/>
+      <c r="Y30" s="76"/>
+      <c r="AB30" s="24"/>
+      <c r="AC30" s="44"/>
+      <c r="AD30" s="24"/>
+      <c r="AE30" s="24"/>
+      <c r="AF30" s="24"/>
+      <c r="AG30" s="24"/>
+      <c r="AH30" s="24"/>
+      <c r="AI30" s="24"/>
+      <c r="BH30" s="70">
+        <v>26</v>
+      </c>
+      <c r="BI30" s="44"/>
+      <c r="BJ30" s="50"/>
+      <c r="BK30" s="52"/>
+      <c r="BL30" s="24"/>
+      <c r="BM30" s="24"/>
     </row>
-    <row r="31" spans="3:35" ht="15" customHeight="1">
-      <c r="N31" s="25"/>
-      <c r="O31" s="26"/>
-      <c r="P31" s="23"/>
-      <c r="Q31" s="26"/>
-      <c r="R31" s="23"/>
-      <c r="S31" s="24"/>
-      <c r="T31" s="21"/>
-      <c r="U31" s="22"/>
-      <c r="V31" s="22"/>
-      <c r="W31" s="22"/>
-      <c r="X31" s="23"/>
-      <c r="Y31" s="24"/>
+    <row r="31" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B31" s="63"/>
+      <c r="C31" s="63"/>
+      <c r="D31" s="63"/>
+      <c r="E31" s="63"/>
+      <c r="F31" s="63"/>
+      <c r="H31" s="63"/>
+      <c r="I31" s="63"/>
+      <c r="J31" s="63"/>
+      <c r="K31" s="63"/>
+      <c r="L31" s="63"/>
+      <c r="M31" s="63"/>
+      <c r="N31" s="76"/>
+      <c r="O31" s="76"/>
+      <c r="P31" s="76"/>
+      <c r="Q31" s="76"/>
+      <c r="R31" s="76"/>
+      <c r="S31" s="76"/>
+      <c r="T31" s="76"/>
+      <c r="U31" s="76"/>
+      <c r="V31" s="76"/>
+      <c r="W31" s="76"/>
+      <c r="X31" s="76"/>
+      <c r="Y31" s="76"/>
+      <c r="AB31" s="24"/>
+      <c r="AC31" s="44"/>
+      <c r="AD31" s="24"/>
+      <c r="AE31" s="24"/>
+      <c r="AF31" s="24"/>
+      <c r="AG31" s="24"/>
+      <c r="AH31" s="24"/>
+      <c r="AI31" s="24"/>
+      <c r="BH31" s="70">
+        <v>27</v>
+      </c>
+      <c r="BI31" s="44"/>
+      <c r="BJ31" s="50"/>
+      <c r="BK31" s="52"/>
+      <c r="BL31" s="24"/>
+      <c r="BM31" s="24"/>
     </row>
-    <row r="32" spans="3:35" ht="15" customHeight="1">
-      <c r="N32" s="25"/>
-      <c r="O32" s="26"/>
-      <c r="P32" s="23"/>
-      <c r="Q32" s="26"/>
-      <c r="R32" s="23"/>
-      <c r="S32" s="24"/>
-      <c r="T32" s="21"/>
-      <c r="U32" s="22"/>
-      <c r="V32" s="22"/>
-      <c r="W32" s="22"/>
-      <c r="X32" s="23"/>
-      <c r="Y32" s="24"/>
+    <row r="32" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B32" s="63"/>
+      <c r="C32" s="63"/>
+      <c r="D32" s="63"/>
+      <c r="E32" s="63"/>
+      <c r="F32" s="63"/>
+      <c r="G32" s="63"/>
+      <c r="H32" s="63"/>
+      <c r="I32" s="63"/>
+      <c r="J32" s="63"/>
+      <c r="K32" s="63"/>
+      <c r="L32" s="63"/>
+      <c r="M32" s="63"/>
+      <c r="N32" s="76"/>
+      <c r="O32" s="76"/>
+      <c r="P32" s="76"/>
+      <c r="Q32" s="76"/>
+      <c r="R32" s="76"/>
+      <c r="S32" s="76"/>
+      <c r="T32" s="76"/>
+      <c r="U32" s="76"/>
+      <c r="V32" s="76"/>
+      <c r="W32" s="76"/>
+      <c r="X32" s="76"/>
+      <c r="Y32" s="76"/>
+      <c r="AB32" s="24"/>
+      <c r="AC32" s="44"/>
+      <c r="AD32" s="24"/>
+      <c r="AE32" s="24"/>
+      <c r="AF32" s="24"/>
+      <c r="AG32" s="24"/>
+      <c r="AH32" s="24"/>
+      <c r="AI32" s="24"/>
+      <c r="BH32" s="70">
+        <v>28</v>
+      </c>
+      <c r="BI32" s="44"/>
+      <c r="BJ32" s="50"/>
+      <c r="BK32" s="52"/>
+      <c r="BL32" s="24"/>
+      <c r="BM32" s="24"/>
     </row>
-    <row r="33" spans="14:25" ht="15" customHeight="1">
-      <c r="N33" s="25"/>
-      <c r="O33" s="26"/>
-      <c r="P33" s="23"/>
-      <c r="Q33" s="26"/>
-      <c r="R33" s="23"/>
-      <c r="S33" s="24"/>
-      <c r="T33" s="21"/>
-      <c r="U33" s="22"/>
-      <c r="V33" s="22"/>
-      <c r="W33" s="22"/>
-      <c r="X33" s="23"/>
-      <c r="Y33" s="24"/>
+    <row r="33" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B33" s="63"/>
+      <c r="C33" s="63"/>
+      <c r="D33" s="63"/>
+      <c r="E33" s="63"/>
+      <c r="F33" s="63"/>
+      <c r="G33" s="63"/>
+      <c r="H33" s="63"/>
+      <c r="I33" s="63"/>
+      <c r="J33" s="63"/>
+      <c r="K33" s="63"/>
+      <c r="L33" s="63"/>
+      <c r="M33" s="63"/>
+      <c r="N33" s="76"/>
+      <c r="O33" s="76"/>
+      <c r="P33" s="76"/>
+      <c r="Q33" s="76"/>
+      <c r="R33" s="76"/>
+      <c r="S33" s="76"/>
+      <c r="T33" s="76"/>
+      <c r="U33" s="76"/>
+      <c r="V33" s="76"/>
+      <c r="W33" s="76"/>
+      <c r="X33" s="76"/>
+      <c r="Y33" s="76"/>
+      <c r="AB33" s="24"/>
+      <c r="AC33" s="44"/>
+      <c r="AD33" s="24"/>
+      <c r="AE33" s="24"/>
+      <c r="AF33" s="24"/>
+      <c r="AG33" s="24"/>
+      <c r="AH33" s="24"/>
+      <c r="AI33" s="24"/>
+      <c r="BH33" s="70">
+        <v>29</v>
+      </c>
+      <c r="BI33" s="44"/>
+      <c r="BJ33" s="50"/>
+      <c r="BK33" s="52"/>
+      <c r="BL33" s="24"/>
+      <c r="BM33" s="24"/>
     </row>
-    <row r="34" spans="14:25" ht="15" customHeight="1">
-      <c r="N34" s="25"/>
-      <c r="O34" s="26"/>
-      <c r="P34" s="23"/>
-      <c r="Q34" s="26"/>
-      <c r="R34" s="23"/>
-      <c r="S34" s="24"/>
-      <c r="T34" s="21"/>
-      <c r="U34" s="22"/>
-      <c r="V34" s="22"/>
-      <c r="W34" s="22"/>
-      <c r="X34" s="23"/>
-      <c r="Y34" s="24"/>
+    <row r="34" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="63"/>
+      <c r="C34" s="63"/>
+      <c r="D34" s="63"/>
+      <c r="E34" s="63"/>
+      <c r="F34" s="63"/>
+      <c r="G34" s="63"/>
+      <c r="H34" s="63"/>
+      <c r="I34" s="63"/>
+      <c r="J34" s="63"/>
+      <c r="K34" s="63"/>
+      <c r="L34" s="63"/>
+      <c r="M34" s="63"/>
+      <c r="N34" s="76"/>
+      <c r="O34" s="76"/>
+      <c r="P34" s="76"/>
+      <c r="Q34" s="76"/>
+      <c r="R34" s="76"/>
+      <c r="S34" s="76"/>
+      <c r="T34" s="76"/>
+      <c r="U34" s="76"/>
+      <c r="V34" s="76"/>
+      <c r="W34" s="76"/>
+      <c r="X34" s="76"/>
+      <c r="Y34" s="76"/>
+      <c r="AB34" s="24"/>
+      <c r="AC34" s="44"/>
+      <c r="AD34" s="24"/>
+      <c r="AE34" s="24"/>
+      <c r="AF34" s="24"/>
+      <c r="AG34" s="24"/>
+      <c r="AH34" s="24"/>
+      <c r="AI34" s="24"/>
+      <c r="BH34" s="70">
+        <v>30</v>
+      </c>
+      <c r="BI34" s="44"/>
+      <c r="BJ34" s="50"/>
+      <c r="BK34" s="52"/>
+      <c r="BL34" s="24"/>
+      <c r="BM34" s="24"/>
     </row>
-    <row r="35" spans="14:25" ht="15" customHeight="1">
-      <c r="N35" s="25"/>
-      <c r="O35" s="26"/>
-      <c r="P35" s="23"/>
-      <c r="Q35" s="26"/>
-      <c r="R35" s="23"/>
-      <c r="S35" s="24"/>
-      <c r="T35" s="21"/>
-      <c r="U35" s="22"/>
-      <c r="V35" s="22"/>
-      <c r="W35" s="22"/>
-      <c r="X35" s="23"/>
-      <c r="Y35" s="24"/>
+    <row r="35" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B35" s="63"/>
+      <c r="C35" s="63"/>
+      <c r="D35" s="63"/>
+      <c r="E35" s="63"/>
+      <c r="F35" s="63"/>
+      <c r="G35" s="63"/>
+      <c r="H35" s="63"/>
+      <c r="I35" s="63"/>
+      <c r="J35" s="63"/>
+      <c r="K35" s="63"/>
+      <c r="L35" s="63"/>
+      <c r="M35" s="63"/>
+      <c r="N35" s="76"/>
+      <c r="O35" s="76"/>
+      <c r="P35" s="76"/>
+      <c r="Q35" s="76"/>
+      <c r="R35" s="76"/>
+      <c r="S35" s="76"/>
+      <c r="T35" s="76"/>
+      <c r="U35" s="76"/>
+      <c r="V35" s="76"/>
+      <c r="W35" s="76"/>
+      <c r="X35" s="76"/>
+      <c r="Y35" s="76"/>
+      <c r="AB35" s="24"/>
+      <c r="AC35" s="44"/>
+      <c r="AD35" s="24"/>
+      <c r="AE35" s="24"/>
+      <c r="AF35" s="24"/>
+      <c r="AG35" s="24"/>
+      <c r="AH35" s="24"/>
+      <c r="AI35" s="24"/>
+      <c r="BH35" s="70">
+        <v>31</v>
+      </c>
+      <c r="BI35" s="44"/>
+      <c r="BJ35" s="50"/>
+      <c r="BK35" s="52"/>
+      <c r="BL35" s="24"/>
+      <c r="BM35" s="24"/>
     </row>
-    <row r="36" spans="14:25" ht="15" customHeight="1">
-      <c r="N36" s="25"/>
-      <c r="O36" s="26"/>
-      <c r="P36" s="23"/>
-      <c r="Q36" s="26"/>
-      <c r="R36" s="23"/>
-      <c r="S36" s="24"/>
-      <c r="T36" s="21"/>
-      <c r="U36" s="22"/>
-      <c r="V36" s="22"/>
-      <c r="W36" s="22"/>
-      <c r="X36" s="23"/>
-      <c r="Y36" s="24"/>
+    <row r="36" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B36" s="63"/>
+      <c r="C36" s="63"/>
+      <c r="D36" s="63"/>
+      <c r="E36" s="63"/>
+      <c r="F36" s="63"/>
+      <c r="G36" s="63"/>
+      <c r="H36" s="63"/>
+      <c r="I36" s="63"/>
+      <c r="J36" s="63"/>
+      <c r="K36" s="63"/>
+      <c r="L36" s="63"/>
+      <c r="M36" s="63"/>
+      <c r="N36" s="76"/>
+      <c r="O36" s="76"/>
+      <c r="P36" s="76"/>
+      <c r="Q36" s="76"/>
+      <c r="R36" s="76"/>
+      <c r="S36" s="76"/>
+      <c r="T36" s="76"/>
+      <c r="U36" s="76"/>
+      <c r="V36" s="76"/>
+      <c r="W36" s="76"/>
+      <c r="X36" s="76"/>
+      <c r="Y36" s="76"/>
+      <c r="AB36" s="24"/>
+      <c r="AC36" s="44"/>
+      <c r="AD36" s="24"/>
+      <c r="AE36" s="24"/>
+      <c r="AF36" s="24"/>
+      <c r="AG36" s="24"/>
+      <c r="AH36" s="24"/>
+      <c r="AI36" s="24"/>
+      <c r="BH36" s="70">
+        <v>32</v>
+      </c>
+      <c r="BI36" s="44"/>
+      <c r="BJ36" s="50"/>
+      <c r="BK36" s="52"/>
+      <c r="BL36" s="24"/>
+      <c r="BM36" s="24"/>
     </row>
-    <row r="37" spans="14:25" ht="15" customHeight="1">
-      <c r="N37" s="25"/>
-      <c r="O37" s="26"/>
-      <c r="P37" s="23"/>
-      <c r="Q37" s="26"/>
-      <c r="R37" s="23"/>
-      <c r="S37" s="24"/>
-      <c r="T37" s="21"/>
-      <c r="U37" s="22"/>
-      <c r="V37" s="22"/>
-      <c r="W37" s="22"/>
-      <c r="X37" s="23"/>
-      <c r="Y37" s="24"/>
+    <row r="37" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B37" s="63"/>
+      <c r="C37" s="63"/>
+      <c r="D37" s="63"/>
+      <c r="E37" s="63"/>
+      <c r="F37" s="63"/>
+      <c r="G37" s="63"/>
+      <c r="H37" s="63"/>
+      <c r="I37" s="63"/>
+      <c r="J37" s="63"/>
+      <c r="K37" s="63"/>
+      <c r="L37" s="63"/>
+      <c r="M37" s="63"/>
+      <c r="N37" s="76"/>
+      <c r="O37" s="76"/>
+      <c r="P37" s="76"/>
+      <c r="Q37" s="76"/>
+      <c r="R37" s="76"/>
+      <c r="S37" s="76"/>
+      <c r="T37" s="76"/>
+      <c r="U37" s="76"/>
+      <c r="V37" s="76"/>
+      <c r="W37" s="76"/>
+      <c r="X37" s="76"/>
+      <c r="Y37" s="76"/>
+      <c r="AB37" s="24"/>
+      <c r="AC37" s="44"/>
+      <c r="AD37" s="24"/>
+      <c r="AE37" s="24"/>
+      <c r="AF37" s="24"/>
+      <c r="AG37" s="24"/>
+      <c r="AH37" s="24"/>
+      <c r="AI37" s="24"/>
+      <c r="BH37" s="70">
+        <v>33</v>
+      </c>
+      <c r="BI37" s="44"/>
+      <c r="BJ37" s="50"/>
+      <c r="BK37" s="52"/>
+      <c r="BL37" s="24"/>
+      <c r="BM37" s="24"/>
     </row>
-    <row r="38" spans="14:25" ht="15" customHeight="1">
-      <c r="N38" s="25"/>
-      <c r="O38" s="26"/>
-      <c r="P38" s="23"/>
-      <c r="Q38" s="26"/>
-      <c r="R38" s="23"/>
-      <c r="S38" s="24"/>
-      <c r="T38" s="21"/>
-      <c r="U38" s="22"/>
-      <c r="V38" s="22"/>
-      <c r="W38" s="22"/>
-      <c r="X38" s="23"/>
-      <c r="Y38" s="24"/>
+    <row r="38" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B38" s="63"/>
+      <c r="C38" s="63"/>
+      <c r="D38" s="63"/>
+      <c r="E38" s="63"/>
+      <c r="F38" s="63"/>
+      <c r="G38" s="63"/>
+      <c r="H38" s="63"/>
+      <c r="I38" s="63"/>
+      <c r="J38" s="63"/>
+      <c r="K38" s="63"/>
+      <c r="L38" s="63"/>
+      <c r="M38" s="63"/>
+      <c r="N38" s="76"/>
+      <c r="O38" s="76"/>
+      <c r="P38" s="76"/>
+      <c r="Q38" s="76"/>
+      <c r="R38" s="76"/>
+      <c r="S38" s="76"/>
+      <c r="T38" s="76"/>
+      <c r="U38" s="76"/>
+      <c r="V38" s="76"/>
+      <c r="W38" s="76"/>
+      <c r="X38" s="76"/>
+      <c r="Y38" s="76"/>
+      <c r="AB38" s="24"/>
+      <c r="AC38" s="44"/>
+      <c r="AD38" s="24"/>
+      <c r="AE38" s="24"/>
+      <c r="AF38" s="24"/>
+      <c r="AG38" s="24"/>
+      <c r="AH38" s="24"/>
+      <c r="AI38" s="24"/>
     </row>
-    <row r="39" spans="14:25" ht="15" customHeight="1">
-      <c r="N39" s="25"/>
-      <c r="O39" s="26"/>
-      <c r="P39" s="23"/>
-      <c r="Q39" s="26"/>
-      <c r="R39" s="23"/>
-      <c r="S39" s="24"/>
-      <c r="T39" s="21"/>
-      <c r="U39" s="22"/>
-      <c r="V39" s="22"/>
-      <c r="W39" s="22"/>
-      <c r="X39" s="23"/>
-      <c r="Y39" s="24"/>
+    <row r="39" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B39" s="63"/>
+      <c r="C39" s="63"/>
+      <c r="D39" s="63"/>
+      <c r="E39" s="63"/>
+      <c r="F39" s="63"/>
+      <c r="G39" s="63"/>
+      <c r="H39" s="63"/>
+      <c r="I39" s="63"/>
+      <c r="J39" s="63"/>
+      <c r="K39" s="63"/>
+      <c r="L39" s="63"/>
+      <c r="M39" s="63"/>
+      <c r="N39" s="76"/>
+      <c r="O39" s="76"/>
+      <c r="P39" s="76"/>
+      <c r="Q39" s="76"/>
+      <c r="R39" s="76"/>
+      <c r="S39" s="76"/>
+      <c r="T39" s="76"/>
+      <c r="U39" s="76"/>
+      <c r="V39" s="76"/>
+      <c r="W39" s="76"/>
+      <c r="X39" s="76"/>
+      <c r="Y39" s="76"/>
+      <c r="AB39" s="24"/>
+      <c r="AC39" s="44"/>
+      <c r="AD39" s="24"/>
+      <c r="AE39" s="24"/>
+      <c r="AF39" s="24"/>
+      <c r="AG39" s="24"/>
+      <c r="AH39" s="24"/>
+      <c r="AI39" s="24"/>
     </row>
-    <row r="40" spans="14:25" ht="15" customHeight="1">
-      <c r="N40" s="25"/>
-      <c r="O40" s="26"/>
-      <c r="P40" s="23"/>
-      <c r="Q40" s="26"/>
-      <c r="R40" s="23"/>
-      <c r="S40" s="24"/>
-      <c r="T40" s="21"/>
-      <c r="U40" s="22"/>
-      <c r="V40" s="22"/>
-      <c r="W40" s="22"/>
-      <c r="X40" s="23"/>
-      <c r="Y40" s="24"/>
+    <row r="40" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B40" s="63"/>
+      <c r="C40" s="63"/>
+      <c r="D40" s="63"/>
+      <c r="E40" s="63"/>
+      <c r="F40" s="63"/>
+      <c r="G40" s="63"/>
+      <c r="H40" s="63"/>
+      <c r="I40" s="63"/>
+      <c r="J40" s="63"/>
+      <c r="K40" s="63"/>
+      <c r="L40" s="63"/>
+      <c r="M40" s="63"/>
+      <c r="N40" s="76"/>
+      <c r="O40" s="76"/>
+      <c r="P40" s="76"/>
+      <c r="Q40" s="76"/>
+      <c r="R40" s="76"/>
+      <c r="S40" s="76"/>
+      <c r="T40" s="76"/>
+      <c r="U40" s="76"/>
+      <c r="V40" s="76"/>
+      <c r="W40" s="76"/>
+      <c r="X40" s="76"/>
+      <c r="Y40" s="76"/>
+      <c r="Z40" s="63"/>
+      <c r="AB40" s="24"/>
+      <c r="AC40" s="44"/>
+      <c r="AD40" s="24"/>
+      <c r="AE40" s="24"/>
+      <c r="AF40" s="24"/>
+      <c r="AG40" s="24"/>
+      <c r="AH40" s="24"/>
+      <c r="AI40" s="24"/>
+    </row>
+    <row r="41" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C41" s="63"/>
+      <c r="D41" s="63"/>
+      <c r="E41" s="63"/>
+      <c r="F41" s="63"/>
+      <c r="G41" s="63"/>
+      <c r="H41" s="63"/>
+      <c r="I41" s="63"/>
+      <c r="J41" s="63"/>
+      <c r="K41" s="63"/>
+      <c r="L41" s="63"/>
+      <c r="M41" s="63"/>
+      <c r="N41" s="76"/>
+      <c r="O41" s="76"/>
+      <c r="P41" s="76"/>
+      <c r="Q41" s="76"/>
+      <c r="R41" s="76"/>
+      <c r="S41" s="76"/>
+      <c r="T41" s="75"/>
+      <c r="U41" s="75"/>
+      <c r="V41" s="75"/>
+      <c r="W41" s="75"/>
+      <c r="X41" s="75"/>
+      <c r="Y41" s="75"/>
+      <c r="Z41" s="63"/>
+    </row>
+    <row r="42" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C42" s="63"/>
+      <c r="D42" s="63"/>
+      <c r="E42" s="63"/>
+      <c r="F42" s="63"/>
+      <c r="G42" s="63"/>
+      <c r="H42" s="63"/>
+      <c r="I42" s="63"/>
+      <c r="J42" s="63"/>
+      <c r="K42" s="63"/>
+      <c r="L42" s="63"/>
+      <c r="M42" s="63"/>
+      <c r="N42" s="76"/>
+      <c r="O42" s="76"/>
+      <c r="P42" s="76"/>
+      <c r="Q42" s="76"/>
+      <c r="R42" s="76"/>
+      <c r="S42" s="76"/>
+      <c r="T42" s="76"/>
+      <c r="U42" s="76"/>
+      <c r="V42" s="76"/>
+      <c r="W42" s="76"/>
+      <c r="X42" s="76"/>
+      <c r="Y42" s="76"/>
+      <c r="Z42" s="63"/>
+    </row>
+    <row r="43" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C43" s="63"/>
+      <c r="D43" s="63"/>
+      <c r="E43" s="63"/>
+      <c r="F43" s="63"/>
+      <c r="G43" s="63"/>
+      <c r="H43" s="63"/>
+      <c r="I43" s="63"/>
+      <c r="J43" s="63"/>
+      <c r="K43" s="63"/>
+      <c r="L43" s="63"/>
+      <c r="M43" s="63"/>
+      <c r="N43" s="76"/>
+      <c r="O43" s="76"/>
+      <c r="P43" s="76"/>
+      <c r="Q43" s="76"/>
+      <c r="R43" s="76"/>
+      <c r="S43" s="76"/>
+      <c r="T43" s="76"/>
+      <c r="U43" s="76"/>
+      <c r="V43" s="76"/>
+      <c r="W43" s="76"/>
+      <c r="X43" s="76"/>
+      <c r="Y43" s="76"/>
+      <c r="Z43" s="63"/>
+    </row>
+    <row r="44" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C44" s="63"/>
+      <c r="D44" s="63"/>
+      <c r="E44" s="63"/>
+      <c r="F44" s="63"/>
+      <c r="G44" s="63"/>
+      <c r="H44" s="63"/>
+      <c r="I44" s="63"/>
+      <c r="J44" s="63"/>
+      <c r="K44" s="63"/>
+      <c r="L44" s="63"/>
+      <c r="M44" s="63"/>
+      <c r="N44" s="76"/>
+      <c r="O44" s="76"/>
+      <c r="P44" s="76"/>
+      <c r="Q44" s="76"/>
+      <c r="R44" s="76"/>
+      <c r="S44" s="76"/>
+      <c r="T44" s="76"/>
+      <c r="U44" s="76"/>
+      <c r="V44" s="76"/>
+      <c r="W44" s="76"/>
+      <c r="X44" s="76"/>
+      <c r="Y44" s="76"/>
+      <c r="Z44" s="63"/>
+    </row>
+    <row r="45" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C45" s="63"/>
+      <c r="D45" s="63"/>
+      <c r="E45" s="63"/>
+      <c r="F45" s="63"/>
+      <c r="G45" s="63"/>
+      <c r="H45" s="63"/>
+      <c r="I45" s="63"/>
+      <c r="J45" s="63"/>
+      <c r="K45" s="63"/>
+      <c r="L45" s="63"/>
+      <c r="M45" s="63"/>
+      <c r="N45" s="76"/>
+      <c r="O45" s="76"/>
+      <c r="P45" s="76"/>
+      <c r="Q45" s="76"/>
+      <c r="R45" s="76"/>
+      <c r="S45" s="76"/>
+      <c r="T45" s="76"/>
+      <c r="U45" s="76"/>
+      <c r="V45" s="76"/>
+      <c r="W45" s="76"/>
+      <c r="X45" s="76"/>
+      <c r="Y45" s="76"/>
+      <c r="Z45" s="63"/>
+    </row>
+    <row r="46" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C46" s="63"/>
+      <c r="D46" s="63"/>
+      <c r="E46" s="63"/>
+      <c r="F46" s="63"/>
+      <c r="G46" s="63"/>
+      <c r="H46" s="63"/>
+      <c r="I46" s="63"/>
+      <c r="J46" s="63"/>
+      <c r="K46" s="63"/>
+      <c r="L46" s="63"/>
+      <c r="M46" s="63"/>
+      <c r="N46" s="76"/>
+      <c r="O46" s="76"/>
+      <c r="P46" s="76"/>
+      <c r="Q46" s="76"/>
+      <c r="R46" s="76"/>
+      <c r="S46" s="76"/>
+      <c r="T46" s="76"/>
+      <c r="U46" s="76"/>
+      <c r="V46" s="76"/>
+      <c r="W46" s="76"/>
+      <c r="X46" s="76"/>
+      <c r="Y46" s="76"/>
+      <c r="Z46" s="63"/>
+    </row>
+    <row r="47" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C47" s="63"/>
+      <c r="D47" s="63"/>
+      <c r="E47" s="63"/>
+      <c r="F47" s="63"/>
+      <c r="G47" s="63"/>
+      <c r="H47" s="63"/>
+      <c r="I47" s="63"/>
+      <c r="J47" s="63"/>
+      <c r="K47" s="63"/>
+      <c r="L47" s="63"/>
+      <c r="M47" s="63"/>
+      <c r="N47" s="76"/>
+      <c r="O47" s="76"/>
+      <c r="P47" s="76"/>
+      <c r="Q47" s="76"/>
+      <c r="R47" s="76"/>
+      <c r="S47" s="76"/>
+      <c r="T47" s="76"/>
+      <c r="U47" s="76"/>
+      <c r="V47" s="76"/>
+      <c r="W47" s="76"/>
+      <c r="X47" s="76"/>
+      <c r="Y47" s="76"/>
+      <c r="Z47" s="63"/>
+    </row>
+    <row r="48" spans="2:65" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C48" s="63"/>
+      <c r="D48" s="63"/>
+      <c r="E48" s="63"/>
+      <c r="F48" s="63"/>
+      <c r="G48" s="63"/>
+      <c r="H48" s="63"/>
+      <c r="I48" s="63"/>
+      <c r="J48" s="63"/>
+      <c r="K48" s="63"/>
+      <c r="L48" s="63"/>
+      <c r="M48" s="63"/>
+      <c r="N48" s="76"/>
+      <c r="O48" s="76"/>
+      <c r="P48" s="76"/>
+      <c r="Q48" s="76"/>
+      <c r="R48" s="76"/>
+      <c r="S48" s="76"/>
+      <c r="T48" s="76"/>
+      <c r="U48" s="76"/>
+      <c r="V48" s="76"/>
+      <c r="W48" s="76"/>
+      <c r="X48" s="76"/>
+      <c r="Y48" s="76"/>
+      <c r="Z48" s="63"/>
+    </row>
+    <row r="49" spans="3:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C49" s="63"/>
+      <c r="D49" s="63"/>
+      <c r="E49" s="63"/>
+      <c r="F49" s="63"/>
+      <c r="G49" s="63"/>
+      <c r="H49" s="63"/>
+      <c r="I49" s="63"/>
+      <c r="J49" s="63"/>
+      <c r="K49" s="63"/>
+      <c r="L49" s="63"/>
+      <c r="M49" s="63"/>
+      <c r="N49" s="76"/>
+      <c r="O49" s="76"/>
+      <c r="P49" s="76"/>
+      <c r="Q49" s="76"/>
+      <c r="R49" s="76"/>
+      <c r="S49" s="76"/>
+      <c r="T49" s="76"/>
+      <c r="U49" s="76"/>
+      <c r="V49" s="76"/>
+      <c r="W49" s="76"/>
+      <c r="X49" s="76"/>
+      <c r="Y49" s="76"/>
+      <c r="Z49" s="63"/>
+    </row>
+    <row r="50" spans="3:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C50" s="63"/>
+      <c r="D50" s="63"/>
+      <c r="E50" s="63"/>
+      <c r="F50" s="63"/>
+      <c r="G50" s="63"/>
+      <c r="H50" s="63"/>
+      <c r="I50" s="63"/>
+      <c r="J50" s="63"/>
+      <c r="K50" s="63"/>
+      <c r="L50" s="63"/>
+      <c r="M50" s="63"/>
+      <c r="N50" s="76"/>
+      <c r="O50" s="76"/>
+      <c r="P50" s="76"/>
+      <c r="Q50" s="76"/>
+      <c r="R50" s="76"/>
+      <c r="S50" s="76"/>
+      <c r="T50" s="76"/>
+      <c r="U50" s="76"/>
+      <c r="V50" s="76"/>
+      <c r="W50" s="76"/>
+      <c r="X50" s="76"/>
+      <c r="Y50" s="76"/>
+      <c r="Z50" s="63"/>
+    </row>
+    <row r="51" spans="3:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C51" s="63"/>
+      <c r="D51" s="63"/>
+      <c r="E51" s="63"/>
+      <c r="F51" s="63"/>
+      <c r="G51" s="63"/>
+      <c r="H51" s="63"/>
+      <c r="I51" s="63"/>
+      <c r="J51" s="63"/>
+      <c r="K51" s="63"/>
+      <c r="L51" s="63"/>
+      <c r="M51" s="63"/>
+      <c r="N51" s="76"/>
+      <c r="O51" s="76"/>
+      <c r="P51" s="76"/>
+      <c r="Q51" s="76"/>
+      <c r="R51" s="76"/>
+      <c r="S51" s="76"/>
+      <c r="T51" s="76"/>
+      <c r="U51" s="76"/>
+      <c r="V51" s="76"/>
+      <c r="W51" s="76"/>
+      <c r="X51" s="76"/>
+      <c r="Y51" s="76"/>
+      <c r="Z51" s="63"/>
+    </row>
+    <row r="52" spans="3:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C52" s="63"/>
+      <c r="D52" s="63"/>
+      <c r="E52" s="63"/>
+      <c r="F52" s="63"/>
+      <c r="G52" s="63"/>
+      <c r="H52" s="63"/>
+      <c r="I52" s="63"/>
+      <c r="J52" s="63"/>
+      <c r="K52" s="63"/>
+      <c r="L52" s="63"/>
+      <c r="M52" s="63"/>
+      <c r="N52" s="76"/>
+      <c r="O52" s="76"/>
+      <c r="P52" s="76"/>
+      <c r="Q52" s="76"/>
+      <c r="R52" s="76"/>
+      <c r="S52" s="76"/>
+      <c r="T52" s="76"/>
+      <c r="U52" s="76"/>
+      <c r="V52" s="76"/>
+      <c r="W52" s="76"/>
+      <c r="X52" s="76"/>
+      <c r="Y52" s="76"/>
+      <c r="Z52" s="63"/>
+    </row>
+    <row r="53" spans="3:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="C53" s="63"/>
+      <c r="D53" s="63"/>
+      <c r="E53" s="63"/>
+      <c r="F53" s="63"/>
+      <c r="G53" s="63"/>
+      <c r="H53" s="63"/>
+      <c r="I53" s="63"/>
+      <c r="J53" s="63"/>
+      <c r="K53" s="63"/>
+      <c r="L53" s="63"/>
+      <c r="M53" s="63"/>
+      <c r="N53" s="76"/>
+      <c r="O53" s="76"/>
+      <c r="P53" s="76"/>
+      <c r="Q53" s="76"/>
+      <c r="R53" s="76"/>
+      <c r="S53" s="76"/>
+      <c r="T53" s="76"/>
+      <c r="U53" s="76"/>
+      <c r="V53" s="76"/>
+      <c r="W53" s="76"/>
+      <c r="X53" s="76"/>
+      <c r="Y53" s="76"/>
+      <c r="Z53" s="63"/>
+    </row>
+    <row r="55" spans="3:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="F55" s="6"/>
+      <c r="G55" s="6"/>
+      <c r="H55" s="6"/>
+      <c r="I55" s="6"/>
+    </row>
+    <row r="56" spans="3:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E56" s="7"/>
+      <c r="J56" s="8"/>
+    </row>
+    <row r="57" spans="3:26" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="E57" s="8"/>
+      <c r="F57" s="6"/>
+      <c r="I57" s="6"/>
+      <c r="J57" s="7"/>
+    </row>
+    <row r="58" spans="3:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F58" s="9"/>
+      <c r="I58" s="11"/>
+    </row>
+    <row r="59" spans="3:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F59" s="10"/>
+      <c r="I59" s="12"/>
+    </row>
+    <row r="60" spans="3:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F60" s="10"/>
+      <c r="I60" s="12"/>
+    </row>
+    <row r="61" spans="3:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F61" s="10"/>
+      <c r="I61" s="12"/>
+    </row>
+    <row r="62" spans="3:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="F62" s="10"/>
+      <c r="I62" s="12"/>
+    </row>
+    <row r="63" spans="3:26" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G63" s="8"/>
+      <c r="H63" s="7"/>
     </row>
   </sheetData>
-  <mergeCells count="323">
-    <mergeCell ref="N10:O10"/>
-    <mergeCell ref="N11:O11"/>
-    <mergeCell ref="N12:O12"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="N14:O14"/>
-    <mergeCell ref="P14:Q14"/>
-    <mergeCell ref="P13:Q13"/>
-    <mergeCell ref="P12:Q12"/>
-    <mergeCell ref="P11:Q11"/>
-    <mergeCell ref="G13:H13"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="P3:Q3"/>
-    <mergeCell ref="R3:S3"/>
-    <mergeCell ref="R4:S4"/>
-    <mergeCell ref="R5:S5"/>
-    <mergeCell ref="R6:S6"/>
-    <mergeCell ref="P10:Q10"/>
-    <mergeCell ref="P9:Q9"/>
-    <mergeCell ref="P8:Q8"/>
-    <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="P5:Q5"/>
-    <mergeCell ref="R13:S13"/>
+  <mergeCells count="442">
+    <mergeCell ref="AB24:AC24"/>
+    <mergeCell ref="AD24:AE24"/>
+    <mergeCell ref="AF24:AG24"/>
+    <mergeCell ref="AH24:AI24"/>
+    <mergeCell ref="AB16:AC16"/>
+    <mergeCell ref="AD16:AE16"/>
+    <mergeCell ref="AF16:AG16"/>
+    <mergeCell ref="AH16:AI16"/>
+    <mergeCell ref="AB11:AI11"/>
+    <mergeCell ref="AB3:AI3"/>
+    <mergeCell ref="AB19:AI19"/>
+    <mergeCell ref="AB22:AC22"/>
+    <mergeCell ref="AD22:AE22"/>
+    <mergeCell ref="BH35:BI35"/>
+    <mergeCell ref="BJ35:BK35"/>
+    <mergeCell ref="BL35:BM35"/>
+    <mergeCell ref="BH36:BI36"/>
+    <mergeCell ref="BJ36:BK36"/>
+    <mergeCell ref="BL36:BM36"/>
+    <mergeCell ref="BH37:BI37"/>
+    <mergeCell ref="BJ37:BK37"/>
+    <mergeCell ref="BL37:BM37"/>
+    <mergeCell ref="BH32:BI32"/>
+    <mergeCell ref="BJ32:BK32"/>
+    <mergeCell ref="BL32:BM32"/>
+    <mergeCell ref="BH33:BI33"/>
+    <mergeCell ref="BJ33:BK33"/>
+    <mergeCell ref="BL33:BM33"/>
+    <mergeCell ref="BH34:BI34"/>
+    <mergeCell ref="BJ34:BK34"/>
+    <mergeCell ref="BL34:BM34"/>
+    <mergeCell ref="BH29:BI29"/>
+    <mergeCell ref="BJ29:BK29"/>
+    <mergeCell ref="BL29:BM29"/>
+    <mergeCell ref="BH30:BI30"/>
+    <mergeCell ref="BJ30:BK30"/>
+    <mergeCell ref="BL30:BM30"/>
+    <mergeCell ref="BH31:BI31"/>
+    <mergeCell ref="BJ31:BK31"/>
+    <mergeCell ref="BL31:BM31"/>
+    <mergeCell ref="BH26:BI26"/>
+    <mergeCell ref="BJ26:BK26"/>
+    <mergeCell ref="BL26:BM26"/>
+    <mergeCell ref="BH27:BI27"/>
+    <mergeCell ref="BJ27:BK27"/>
+    <mergeCell ref="BL27:BM27"/>
+    <mergeCell ref="BH28:BI28"/>
+    <mergeCell ref="BJ28:BK28"/>
+    <mergeCell ref="BL28:BM28"/>
+    <mergeCell ref="BH23:BI23"/>
+    <mergeCell ref="BJ23:BK23"/>
+    <mergeCell ref="BL23:BM23"/>
+    <mergeCell ref="BH24:BI24"/>
+    <mergeCell ref="BJ24:BK24"/>
+    <mergeCell ref="BL24:BM24"/>
+    <mergeCell ref="BH25:BI25"/>
+    <mergeCell ref="BJ25:BK25"/>
+    <mergeCell ref="BL25:BM25"/>
+    <mergeCell ref="BH19:BI19"/>
+    <mergeCell ref="BJ19:BK19"/>
+    <mergeCell ref="BL19:BM19"/>
+    <mergeCell ref="BH20:BI20"/>
+    <mergeCell ref="BJ20:BK20"/>
+    <mergeCell ref="BL20:BM20"/>
+    <mergeCell ref="BH22:BI22"/>
+    <mergeCell ref="BJ22:BK22"/>
+    <mergeCell ref="BL22:BM22"/>
+    <mergeCell ref="BH21:BI21"/>
+    <mergeCell ref="BJ21:BK21"/>
+    <mergeCell ref="BL21:BM21"/>
+    <mergeCell ref="BH16:BI16"/>
+    <mergeCell ref="BJ16:BK16"/>
+    <mergeCell ref="BL16:BM16"/>
+    <mergeCell ref="BH18:BI18"/>
+    <mergeCell ref="BJ18:BK18"/>
+    <mergeCell ref="BL18:BM18"/>
+    <mergeCell ref="BH17:BI17"/>
+    <mergeCell ref="BJ17:BK17"/>
+    <mergeCell ref="BL17:BM17"/>
+    <mergeCell ref="BJ12:BK12"/>
+    <mergeCell ref="BL12:BM12"/>
+    <mergeCell ref="BH13:BI13"/>
+    <mergeCell ref="BJ13:BK13"/>
+    <mergeCell ref="BL13:BM13"/>
+    <mergeCell ref="BH14:BI14"/>
+    <mergeCell ref="BJ14:BK14"/>
+    <mergeCell ref="BL14:BM14"/>
+    <mergeCell ref="BH15:BI15"/>
+    <mergeCell ref="BJ15:BK15"/>
+    <mergeCell ref="BL15:BM15"/>
+    <mergeCell ref="BJ8:BK8"/>
+    <mergeCell ref="BL8:BM8"/>
+    <mergeCell ref="BH9:BI9"/>
+    <mergeCell ref="BJ9:BK9"/>
+    <mergeCell ref="BL9:BM9"/>
+    <mergeCell ref="BH10:BI10"/>
+    <mergeCell ref="BJ10:BK10"/>
+    <mergeCell ref="BL10:BM10"/>
+    <mergeCell ref="BH11:BI11"/>
+    <mergeCell ref="BJ11:BK11"/>
+    <mergeCell ref="BL11:BM11"/>
+    <mergeCell ref="BJ4:BK4"/>
+    <mergeCell ref="BL4:BM4"/>
+    <mergeCell ref="BH5:BI5"/>
+    <mergeCell ref="BJ5:BK5"/>
+    <mergeCell ref="BL5:BM5"/>
+    <mergeCell ref="BH6:BI6"/>
+    <mergeCell ref="BJ6:BK6"/>
+    <mergeCell ref="BL6:BM6"/>
+    <mergeCell ref="BH7:BI7"/>
+    <mergeCell ref="BJ7:BK7"/>
+    <mergeCell ref="BL7:BM7"/>
+    <mergeCell ref="AL13:AM13"/>
+    <mergeCell ref="AN13:AO13"/>
+    <mergeCell ref="AP13:AQ13"/>
+    <mergeCell ref="AR13:AS13"/>
+    <mergeCell ref="AL14:AM14"/>
+    <mergeCell ref="AN14:AO14"/>
+    <mergeCell ref="AP14:AQ14"/>
+    <mergeCell ref="AR14:AS14"/>
+    <mergeCell ref="BH4:BI4"/>
+    <mergeCell ref="BH8:BI8"/>
+    <mergeCell ref="BH12:BI12"/>
+    <mergeCell ref="AL10:AM10"/>
+    <mergeCell ref="AN10:AO10"/>
+    <mergeCell ref="AP10:AQ10"/>
+    <mergeCell ref="AR10:AS10"/>
+    <mergeCell ref="AL11:AM11"/>
+    <mergeCell ref="AN11:AO11"/>
+    <mergeCell ref="AP11:AQ11"/>
+    <mergeCell ref="AR11:AS11"/>
+    <mergeCell ref="AL12:AM12"/>
+    <mergeCell ref="AN12:AO12"/>
+    <mergeCell ref="AP12:AQ12"/>
+    <mergeCell ref="AR12:AS12"/>
+    <mergeCell ref="AL7:AM7"/>
+    <mergeCell ref="AN7:AO7"/>
+    <mergeCell ref="AP7:AQ7"/>
+    <mergeCell ref="AR7:AS7"/>
+    <mergeCell ref="AL8:AM8"/>
+    <mergeCell ref="AN8:AO8"/>
+    <mergeCell ref="AP8:AQ8"/>
+    <mergeCell ref="AR8:AS8"/>
+    <mergeCell ref="AL9:AM9"/>
+    <mergeCell ref="AN9:AO9"/>
+    <mergeCell ref="AP9:AQ9"/>
+    <mergeCell ref="AR9:AS9"/>
+    <mergeCell ref="AL4:AM4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AP4:AQ4"/>
+    <mergeCell ref="AR4:AS4"/>
+    <mergeCell ref="AL5:AM5"/>
+    <mergeCell ref="AN5:AO5"/>
+    <mergeCell ref="AP5:AQ5"/>
+    <mergeCell ref="AR5:AS5"/>
+    <mergeCell ref="AL6:AM6"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AP6:AQ6"/>
+    <mergeCell ref="AR6:AS6"/>
+    <mergeCell ref="BH3:BI3"/>
+    <mergeCell ref="BH2:BM2"/>
+    <mergeCell ref="BJ3:BK3"/>
+    <mergeCell ref="BL3:BM3"/>
+    <mergeCell ref="AL2:AS2"/>
+    <mergeCell ref="AL3:AM3"/>
+    <mergeCell ref="AN3:AO3"/>
+    <mergeCell ref="AP3:AQ3"/>
+    <mergeCell ref="AR3:AS3"/>
+    <mergeCell ref="AH38:AI38"/>
+    <mergeCell ref="AB39:AC39"/>
+    <mergeCell ref="AD39:AE39"/>
+    <mergeCell ref="AF39:AG39"/>
+    <mergeCell ref="AH39:AI39"/>
+    <mergeCell ref="AB40:AC40"/>
+    <mergeCell ref="AD40:AE40"/>
+    <mergeCell ref="AF40:AG40"/>
+    <mergeCell ref="AH40:AI40"/>
+    <mergeCell ref="AH35:AI35"/>
+    <mergeCell ref="AB36:AC36"/>
+    <mergeCell ref="AD36:AE36"/>
+    <mergeCell ref="AF36:AG36"/>
+    <mergeCell ref="AH36:AI36"/>
+    <mergeCell ref="AB37:AC37"/>
+    <mergeCell ref="AD37:AE37"/>
+    <mergeCell ref="AF37:AG37"/>
+    <mergeCell ref="AH37:AI37"/>
+    <mergeCell ref="AH32:AI32"/>
+    <mergeCell ref="AB33:AC33"/>
+    <mergeCell ref="AD33:AE33"/>
+    <mergeCell ref="AF33:AG33"/>
+    <mergeCell ref="AH33:AI33"/>
+    <mergeCell ref="AB34:AC34"/>
+    <mergeCell ref="AD34:AE34"/>
+    <mergeCell ref="AF34:AG34"/>
+    <mergeCell ref="AH34:AI34"/>
+    <mergeCell ref="AH29:AI29"/>
+    <mergeCell ref="AB30:AC30"/>
+    <mergeCell ref="AD30:AE30"/>
+    <mergeCell ref="AF30:AG30"/>
+    <mergeCell ref="AH30:AI30"/>
+    <mergeCell ref="AB31:AC31"/>
+    <mergeCell ref="AD31:AE31"/>
+    <mergeCell ref="AF31:AG31"/>
+    <mergeCell ref="AH31:AI31"/>
+    <mergeCell ref="AB29:AC29"/>
+    <mergeCell ref="AD29:AE29"/>
+    <mergeCell ref="AF29:AG29"/>
+    <mergeCell ref="AB32:AC32"/>
+    <mergeCell ref="AD32:AE32"/>
+    <mergeCell ref="AF32:AG32"/>
+    <mergeCell ref="AB35:AC35"/>
+    <mergeCell ref="AD35:AE35"/>
+    <mergeCell ref="AF35:AG35"/>
+    <mergeCell ref="AB38:AC38"/>
+    <mergeCell ref="AD38:AE38"/>
+    <mergeCell ref="AF38:AG38"/>
+    <mergeCell ref="G26:H26"/>
+    <mergeCell ref="AB28:AI28"/>
+    <mergeCell ref="AB26:AC26"/>
+    <mergeCell ref="AD26:AE26"/>
+    <mergeCell ref="AF26:AG26"/>
+    <mergeCell ref="AH26:AI26"/>
+    <mergeCell ref="AB27:AC27"/>
+    <mergeCell ref="AD27:AE27"/>
+    <mergeCell ref="AF27:AG27"/>
+    <mergeCell ref="AH27:AI27"/>
+    <mergeCell ref="AF22:AG22"/>
+    <mergeCell ref="AH22:AI22"/>
+    <mergeCell ref="AB23:AC23"/>
+    <mergeCell ref="AD23:AE23"/>
+    <mergeCell ref="AF23:AG23"/>
+    <mergeCell ref="AH23:AI23"/>
+    <mergeCell ref="AB20:AC20"/>
+    <mergeCell ref="AD20:AE20"/>
+    <mergeCell ref="AF20:AG20"/>
+    <mergeCell ref="AH20:AI20"/>
+    <mergeCell ref="AB21:AC21"/>
+    <mergeCell ref="AD21:AE21"/>
+    <mergeCell ref="AF21:AG21"/>
+    <mergeCell ref="AH21:AI21"/>
+    <mergeCell ref="T27:U27"/>
+    <mergeCell ref="V27:W27"/>
+    <mergeCell ref="X27:Y27"/>
+    <mergeCell ref="T15:Y15"/>
+    <mergeCell ref="T25:U25"/>
+    <mergeCell ref="V25:W25"/>
+    <mergeCell ref="X25:Y25"/>
+    <mergeCell ref="T26:U26"/>
+    <mergeCell ref="V26:W26"/>
+    <mergeCell ref="X26:Y26"/>
+    <mergeCell ref="T23:U23"/>
+    <mergeCell ref="V23:W23"/>
+    <mergeCell ref="X23:Y23"/>
+    <mergeCell ref="T24:U24"/>
+    <mergeCell ref="V24:W24"/>
+    <mergeCell ref="X24:Y24"/>
+    <mergeCell ref="T21:U21"/>
+    <mergeCell ref="V21:W21"/>
+    <mergeCell ref="T17:U17"/>
+    <mergeCell ref="V17:W17"/>
+    <mergeCell ref="X17:Y17"/>
+    <mergeCell ref="T18:U18"/>
+    <mergeCell ref="V18:W18"/>
+    <mergeCell ref="X18:Y18"/>
+    <mergeCell ref="T16:U16"/>
+    <mergeCell ref="V16:W16"/>
+    <mergeCell ref="X16:Y16"/>
+    <mergeCell ref="N26:O26"/>
+    <mergeCell ref="P26:Q26"/>
+    <mergeCell ref="R26:S26"/>
+    <mergeCell ref="N27:O27"/>
+    <mergeCell ref="P27:Q27"/>
+    <mergeCell ref="R27:S27"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="P24:Q24"/>
+    <mergeCell ref="R24:S24"/>
+    <mergeCell ref="N25:O25"/>
+    <mergeCell ref="P25:Q25"/>
+    <mergeCell ref="R25:S25"/>
+    <mergeCell ref="N23:O23"/>
+    <mergeCell ref="P23:Q23"/>
+    <mergeCell ref="R23:S23"/>
+    <mergeCell ref="N20:O20"/>
+    <mergeCell ref="P20:Q20"/>
+    <mergeCell ref="R20:S20"/>
+    <mergeCell ref="N21:O21"/>
+    <mergeCell ref="P21:Q21"/>
+    <mergeCell ref="R21:S21"/>
+    <mergeCell ref="R18:S18"/>
+    <mergeCell ref="N19:O19"/>
+    <mergeCell ref="P19:Q19"/>
+    <mergeCell ref="R19:S19"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="P22:Q22"/>
+    <mergeCell ref="R22:S22"/>
+    <mergeCell ref="X21:Y21"/>
+    <mergeCell ref="T22:U22"/>
+    <mergeCell ref="V22:W22"/>
+    <mergeCell ref="X22:Y22"/>
+    <mergeCell ref="T19:U19"/>
+    <mergeCell ref="V19:W19"/>
+    <mergeCell ref="X19:Y19"/>
+    <mergeCell ref="T20:U20"/>
+    <mergeCell ref="V20:W20"/>
+    <mergeCell ref="X20:Y20"/>
+    <mergeCell ref="N15:S15"/>
+    <mergeCell ref="N16:O16"/>
+    <mergeCell ref="P16:Q16"/>
+    <mergeCell ref="R16:S16"/>
+    <mergeCell ref="N17:O17"/>
+    <mergeCell ref="P17:Q17"/>
+    <mergeCell ref="AB18:AC18"/>
+    <mergeCell ref="AD18:AE18"/>
+    <mergeCell ref="AF18:AG18"/>
+    <mergeCell ref="AH18:AI18"/>
+    <mergeCell ref="AB17:AC17"/>
+    <mergeCell ref="AD17:AE17"/>
+    <mergeCell ref="AF17:AG17"/>
+    <mergeCell ref="AH17:AI17"/>
+    <mergeCell ref="R17:S17"/>
+    <mergeCell ref="N18:O18"/>
+    <mergeCell ref="P18:Q18"/>
+    <mergeCell ref="AB14:AC14"/>
+    <mergeCell ref="AD14:AE14"/>
+    <mergeCell ref="AF14:AG14"/>
+    <mergeCell ref="AH14:AI14"/>
+    <mergeCell ref="AB15:AC15"/>
+    <mergeCell ref="AD15:AE15"/>
+    <mergeCell ref="AF15:AG15"/>
+    <mergeCell ref="AH15:AI15"/>
+    <mergeCell ref="AB12:AC12"/>
+    <mergeCell ref="AD12:AE12"/>
+    <mergeCell ref="AF12:AG12"/>
+    <mergeCell ref="AH12:AI12"/>
+    <mergeCell ref="AB13:AC13"/>
+    <mergeCell ref="AD13:AE13"/>
+    <mergeCell ref="AF13:AG13"/>
+    <mergeCell ref="AH13:AI13"/>
+    <mergeCell ref="AF9:AG9"/>
+    <mergeCell ref="AH9:AI9"/>
+    <mergeCell ref="AB10:AC10"/>
+    <mergeCell ref="AD10:AE10"/>
+    <mergeCell ref="AF10:AG10"/>
+    <mergeCell ref="AH10:AI10"/>
+    <mergeCell ref="AB8:AC8"/>
+    <mergeCell ref="AD8:AE8"/>
+    <mergeCell ref="AF8:AG8"/>
+    <mergeCell ref="AH8:AI8"/>
+    <mergeCell ref="AB9:AC9"/>
+    <mergeCell ref="AD9:AE9"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AD6:AE6"/>
+    <mergeCell ref="AF6:AG6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AB7:AC7"/>
+    <mergeCell ref="AD7:AE7"/>
+    <mergeCell ref="AF7:AG7"/>
+    <mergeCell ref="AH7:AI7"/>
+    <mergeCell ref="AD4:AE4"/>
+    <mergeCell ref="AF4:AG4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AB5:AC5"/>
+    <mergeCell ref="AD5:AE5"/>
+    <mergeCell ref="AF5:AG5"/>
+    <mergeCell ref="AH5:AI5"/>
+    <mergeCell ref="T14:U14"/>
+    <mergeCell ref="V14:W14"/>
+    <mergeCell ref="X14:Y14"/>
+    <mergeCell ref="AB2:AI2"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="T12:U12"/>
+    <mergeCell ref="V12:W12"/>
+    <mergeCell ref="X12:Y12"/>
+    <mergeCell ref="T13:U13"/>
+    <mergeCell ref="V13:W13"/>
+    <mergeCell ref="X13:Y13"/>
+    <mergeCell ref="T10:U10"/>
+    <mergeCell ref="V10:W10"/>
+    <mergeCell ref="X10:Y10"/>
+    <mergeCell ref="T11:U11"/>
+    <mergeCell ref="V11:W11"/>
+    <mergeCell ref="X11:Y11"/>
+    <mergeCell ref="T8:U8"/>
+    <mergeCell ref="V8:W8"/>
+    <mergeCell ref="X8:Y8"/>
+    <mergeCell ref="V9:W9"/>
+    <mergeCell ref="X9:Y9"/>
+    <mergeCell ref="V5:W5"/>
+    <mergeCell ref="X5:Y5"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="X6:Y6"/>
+    <mergeCell ref="T7:U7"/>
+    <mergeCell ref="V7:W7"/>
+    <mergeCell ref="X7:Y7"/>
     <mergeCell ref="R14:S14"/>
     <mergeCell ref="T2:Y2"/>
     <mergeCell ref="T3:U3"/>
@@ -4546,282 +6210,29 @@
     <mergeCell ref="N8:O8"/>
     <mergeCell ref="N9:O9"/>
     <mergeCell ref="T9:U9"/>
-    <mergeCell ref="V9:W9"/>
-    <mergeCell ref="X9:Y9"/>
-    <mergeCell ref="V5:W5"/>
-    <mergeCell ref="X5:Y5"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="X6:Y6"/>
-    <mergeCell ref="T7:U7"/>
-    <mergeCell ref="V7:W7"/>
-    <mergeCell ref="X7:Y7"/>
-    <mergeCell ref="T14:U14"/>
-    <mergeCell ref="V14:W14"/>
-    <mergeCell ref="X14:Y14"/>
-    <mergeCell ref="AB3:AC3"/>
-    <mergeCell ref="AD3:AE3"/>
-    <mergeCell ref="AB2:AI2"/>
-    <mergeCell ref="AF3:AG3"/>
-    <mergeCell ref="AH3:AI3"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="T12:U12"/>
-    <mergeCell ref="V12:W12"/>
-    <mergeCell ref="X12:Y12"/>
-    <mergeCell ref="T13:U13"/>
-    <mergeCell ref="V13:W13"/>
-    <mergeCell ref="X13:Y13"/>
-    <mergeCell ref="T10:U10"/>
-    <mergeCell ref="V10:W10"/>
-    <mergeCell ref="X10:Y10"/>
-    <mergeCell ref="T11:U11"/>
-    <mergeCell ref="V11:W11"/>
-    <mergeCell ref="X11:Y11"/>
-    <mergeCell ref="T8:U8"/>
-    <mergeCell ref="V8:W8"/>
-    <mergeCell ref="X8:Y8"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AD6:AE6"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AB7:AC7"/>
-    <mergeCell ref="AD7:AE7"/>
-    <mergeCell ref="AF7:AG7"/>
-    <mergeCell ref="AH7:AI7"/>
-    <mergeCell ref="AD4:AE4"/>
-    <mergeCell ref="AF4:AG4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AB5:AC5"/>
-    <mergeCell ref="AD5:AE5"/>
-    <mergeCell ref="AF5:AG5"/>
-    <mergeCell ref="AH5:AI5"/>
-    <mergeCell ref="AF9:AG9"/>
-    <mergeCell ref="AH9:AI9"/>
-    <mergeCell ref="AB10:AC10"/>
-    <mergeCell ref="AD10:AE10"/>
-    <mergeCell ref="AF10:AG10"/>
-    <mergeCell ref="AH10:AI10"/>
-    <mergeCell ref="AB8:AC8"/>
-    <mergeCell ref="AD8:AE8"/>
-    <mergeCell ref="AF8:AG8"/>
-    <mergeCell ref="AH8:AI8"/>
-    <mergeCell ref="AB9:AC9"/>
-    <mergeCell ref="AD9:AE9"/>
-    <mergeCell ref="AB13:AC13"/>
-    <mergeCell ref="AD13:AE13"/>
-    <mergeCell ref="AF13:AG13"/>
-    <mergeCell ref="AH13:AI13"/>
-    <mergeCell ref="AB14:AC14"/>
-    <mergeCell ref="AD14:AE14"/>
-    <mergeCell ref="AF14:AG14"/>
-    <mergeCell ref="AH14:AI14"/>
-    <mergeCell ref="AB11:AC11"/>
-    <mergeCell ref="AD11:AE11"/>
-    <mergeCell ref="AF11:AG11"/>
-    <mergeCell ref="AH11:AI11"/>
-    <mergeCell ref="AB12:AC12"/>
-    <mergeCell ref="AD12:AE12"/>
-    <mergeCell ref="AF12:AG12"/>
-    <mergeCell ref="AH12:AI12"/>
-    <mergeCell ref="AF19:AG19"/>
-    <mergeCell ref="AH19:AI19"/>
-    <mergeCell ref="N15:S15"/>
-    <mergeCell ref="N16:O16"/>
-    <mergeCell ref="P16:Q16"/>
-    <mergeCell ref="R16:S16"/>
-    <mergeCell ref="N17:O17"/>
-    <mergeCell ref="P17:Q17"/>
-    <mergeCell ref="AB17:AC17"/>
-    <mergeCell ref="AD17:AE17"/>
-    <mergeCell ref="AF17:AG17"/>
-    <mergeCell ref="AH17:AI17"/>
-    <mergeCell ref="AB18:AC18"/>
-    <mergeCell ref="AD18:AE18"/>
-    <mergeCell ref="AF18:AG18"/>
-    <mergeCell ref="AH18:AI18"/>
-    <mergeCell ref="AB16:AC16"/>
-    <mergeCell ref="AD16:AE16"/>
-    <mergeCell ref="AF16:AG16"/>
-    <mergeCell ref="AH16:AI16"/>
-    <mergeCell ref="AB15:AI15"/>
-    <mergeCell ref="R17:S17"/>
-    <mergeCell ref="N18:O18"/>
-    <mergeCell ref="P18:Q18"/>
-    <mergeCell ref="R18:S18"/>
-    <mergeCell ref="N19:O19"/>
-    <mergeCell ref="P19:Q19"/>
-    <mergeCell ref="R19:S19"/>
-    <mergeCell ref="AB19:AC19"/>
-    <mergeCell ref="AD19:AE19"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="P22:Q22"/>
-    <mergeCell ref="R22:S22"/>
-    <mergeCell ref="N23:O23"/>
-    <mergeCell ref="P23:Q23"/>
-    <mergeCell ref="R23:S23"/>
-    <mergeCell ref="N20:O20"/>
-    <mergeCell ref="P20:Q20"/>
-    <mergeCell ref="R20:S20"/>
-    <mergeCell ref="N21:O21"/>
-    <mergeCell ref="P21:Q21"/>
-    <mergeCell ref="R21:S21"/>
-    <mergeCell ref="N26:O26"/>
-    <mergeCell ref="P26:Q26"/>
-    <mergeCell ref="R26:S26"/>
-    <mergeCell ref="N27:O27"/>
-    <mergeCell ref="P27:Q27"/>
-    <mergeCell ref="R27:S27"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="P24:Q24"/>
-    <mergeCell ref="R24:S24"/>
-    <mergeCell ref="N25:O25"/>
-    <mergeCell ref="P25:Q25"/>
-    <mergeCell ref="R25:S25"/>
-    <mergeCell ref="T17:U17"/>
-    <mergeCell ref="V17:W17"/>
-    <mergeCell ref="X17:Y17"/>
-    <mergeCell ref="T18:U18"/>
-    <mergeCell ref="V18:W18"/>
-    <mergeCell ref="X18:Y18"/>
-    <mergeCell ref="T16:U16"/>
-    <mergeCell ref="V16:W16"/>
-    <mergeCell ref="X16:Y16"/>
-    <mergeCell ref="X21:Y21"/>
-    <mergeCell ref="T22:U22"/>
-    <mergeCell ref="V22:W22"/>
-    <mergeCell ref="X22:Y22"/>
-    <mergeCell ref="T19:U19"/>
-    <mergeCell ref="V19:W19"/>
-    <mergeCell ref="X19:Y19"/>
-    <mergeCell ref="T20:U20"/>
-    <mergeCell ref="V20:W20"/>
-    <mergeCell ref="X20:Y20"/>
-    <mergeCell ref="R29:S29"/>
-    <mergeCell ref="N30:O30"/>
-    <mergeCell ref="P30:Q30"/>
-    <mergeCell ref="R30:S30"/>
-    <mergeCell ref="T27:U27"/>
-    <mergeCell ref="V27:W27"/>
-    <mergeCell ref="X27:Y27"/>
-    <mergeCell ref="T15:Y15"/>
-    <mergeCell ref="T28:Y28"/>
-    <mergeCell ref="N28:S28"/>
-    <mergeCell ref="T25:U25"/>
-    <mergeCell ref="V25:W25"/>
-    <mergeCell ref="X25:Y25"/>
-    <mergeCell ref="T26:U26"/>
-    <mergeCell ref="V26:W26"/>
-    <mergeCell ref="X26:Y26"/>
-    <mergeCell ref="T23:U23"/>
-    <mergeCell ref="V23:W23"/>
-    <mergeCell ref="X23:Y23"/>
-    <mergeCell ref="T24:U24"/>
-    <mergeCell ref="V24:W24"/>
-    <mergeCell ref="X24:Y24"/>
-    <mergeCell ref="T21:U21"/>
-    <mergeCell ref="V21:W21"/>
-    <mergeCell ref="AB22:AC22"/>
-    <mergeCell ref="AD22:AE22"/>
-    <mergeCell ref="AF22:AG22"/>
-    <mergeCell ref="AH22:AI22"/>
-    <mergeCell ref="AB23:AC23"/>
-    <mergeCell ref="AD23:AE23"/>
-    <mergeCell ref="AF23:AG23"/>
-    <mergeCell ref="AH23:AI23"/>
-    <mergeCell ref="AB20:AC20"/>
-    <mergeCell ref="AD20:AE20"/>
-    <mergeCell ref="AF20:AG20"/>
-    <mergeCell ref="AH20:AI20"/>
-    <mergeCell ref="AB21:AC21"/>
-    <mergeCell ref="AD21:AE21"/>
-    <mergeCell ref="AF21:AG21"/>
-    <mergeCell ref="AH21:AI21"/>
-    <mergeCell ref="AB26:AC26"/>
-    <mergeCell ref="AD26:AE26"/>
-    <mergeCell ref="AF26:AG26"/>
-    <mergeCell ref="AH26:AI26"/>
-    <mergeCell ref="AB27:AC27"/>
-    <mergeCell ref="AD27:AE27"/>
-    <mergeCell ref="AF27:AG27"/>
-    <mergeCell ref="AH27:AI27"/>
-    <mergeCell ref="AB24:AC24"/>
-    <mergeCell ref="AD24:AE24"/>
-    <mergeCell ref="AF24:AG24"/>
-    <mergeCell ref="AH24:AI24"/>
-    <mergeCell ref="AB25:AC25"/>
-    <mergeCell ref="AD25:AE25"/>
-    <mergeCell ref="AF25:AG25"/>
-    <mergeCell ref="AH25:AI25"/>
-    <mergeCell ref="N35:O35"/>
-    <mergeCell ref="P35:Q35"/>
-    <mergeCell ref="R35:S35"/>
-    <mergeCell ref="N36:O36"/>
-    <mergeCell ref="P36:Q36"/>
-    <mergeCell ref="R36:S36"/>
-    <mergeCell ref="AB28:AI28"/>
-    <mergeCell ref="N33:O33"/>
-    <mergeCell ref="P33:Q33"/>
-    <mergeCell ref="R33:S33"/>
-    <mergeCell ref="N34:O34"/>
-    <mergeCell ref="P34:Q34"/>
-    <mergeCell ref="R34:S34"/>
-    <mergeCell ref="T29:U29"/>
-    <mergeCell ref="V29:W29"/>
-    <mergeCell ref="X29:Y29"/>
-    <mergeCell ref="N31:O31"/>
-    <mergeCell ref="P31:Q31"/>
-    <mergeCell ref="R31:S31"/>
-    <mergeCell ref="N32:O32"/>
-    <mergeCell ref="P32:Q32"/>
-    <mergeCell ref="R32:S32"/>
-    <mergeCell ref="N29:O29"/>
-    <mergeCell ref="P29:Q29"/>
-    <mergeCell ref="N39:O39"/>
-    <mergeCell ref="P39:Q39"/>
-    <mergeCell ref="R39:S39"/>
-    <mergeCell ref="N40:O40"/>
-    <mergeCell ref="P40:Q40"/>
-    <mergeCell ref="R40:S40"/>
-    <mergeCell ref="N37:O37"/>
-    <mergeCell ref="P37:Q37"/>
-    <mergeCell ref="R37:S37"/>
-    <mergeCell ref="N38:O38"/>
-    <mergeCell ref="P38:Q38"/>
-    <mergeCell ref="R38:S38"/>
-    <mergeCell ref="X32:Y32"/>
-    <mergeCell ref="T33:U33"/>
-    <mergeCell ref="V33:W33"/>
-    <mergeCell ref="X33:Y33"/>
-    <mergeCell ref="T30:U30"/>
-    <mergeCell ref="V30:W30"/>
-    <mergeCell ref="X30:Y30"/>
-    <mergeCell ref="T31:U31"/>
-    <mergeCell ref="V31:W31"/>
-    <mergeCell ref="X31:Y31"/>
-    <mergeCell ref="T40:U40"/>
-    <mergeCell ref="V40:W40"/>
-    <mergeCell ref="X40:Y40"/>
-    <mergeCell ref="G26:H26"/>
-    <mergeCell ref="T38:U38"/>
-    <mergeCell ref="V38:W38"/>
-    <mergeCell ref="X38:Y38"/>
-    <mergeCell ref="T39:U39"/>
-    <mergeCell ref="V39:W39"/>
-    <mergeCell ref="X39:Y39"/>
-    <mergeCell ref="T36:U36"/>
-    <mergeCell ref="V36:W36"/>
-    <mergeCell ref="X36:Y36"/>
-    <mergeCell ref="T37:U37"/>
-    <mergeCell ref="V37:W37"/>
-    <mergeCell ref="X37:Y37"/>
-    <mergeCell ref="T34:U34"/>
-    <mergeCell ref="V34:W34"/>
-    <mergeCell ref="X34:Y34"/>
-    <mergeCell ref="T35:U35"/>
-    <mergeCell ref="V35:W35"/>
-    <mergeCell ref="X35:Y35"/>
-    <mergeCell ref="T32:U32"/>
-    <mergeCell ref="V32:W32"/>
+    <mergeCell ref="G13:H13"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="P3:Q3"/>
+    <mergeCell ref="R3:S3"/>
+    <mergeCell ref="R4:S4"/>
+    <mergeCell ref="R5:S5"/>
+    <mergeCell ref="R6:S6"/>
+    <mergeCell ref="P10:Q10"/>
+    <mergeCell ref="P9:Q9"/>
+    <mergeCell ref="P8:Q8"/>
+    <mergeCell ref="P7:Q7"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="P5:Q5"/>
+    <mergeCell ref="R13:S13"/>
+    <mergeCell ref="N10:O10"/>
+    <mergeCell ref="N11:O11"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="N14:O14"/>
+    <mergeCell ref="P14:Q14"/>
+    <mergeCell ref="P13:Q13"/>
+    <mergeCell ref="P12:Q12"/>
+    <mergeCell ref="P11:Q11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>